<commit_message>
voting stats dashboard update
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A0AA4AA-BD6D-4F50-96B9-96E764574BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE713E3-B397-46E3-B014-CFEED9A97C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22944" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1523,9 +1523,6 @@
       <c r="D52" t="s">
         <v>65</v>
       </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -1540,9 +1537,6 @@
       <c r="D53" t="s">
         <v>66</v>
       </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -1557,9 +1551,6 @@
       <c r="D54" t="s">
         <v>67</v>
       </c>
-      <c r="E54">
-        <v>3</v>
-      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
@@ -1574,9 +1565,6 @@
       <c r="D55" t="s">
         <v>68</v>
       </c>
-      <c r="E55">
-        <v>4</v>
-      </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
@@ -1591,9 +1579,6 @@
       <c r="D56" t="s">
         <v>70</v>
       </c>
-      <c r="E56">
-        <v>5</v>
-      </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
@@ -1608,9 +1593,6 @@
       <c r="D57" t="s">
         <v>69</v>
       </c>
-      <c r="E57">
-        <v>6</v>
-      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
@@ -1625,9 +1607,6 @@
       <c r="D58" t="s">
         <v>71</v>
       </c>
-      <c r="E58">
-        <v>7</v>
-      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
@@ -1642,9 +1621,6 @@
       <c r="D59" t="s">
         <v>72</v>
       </c>
-      <c r="E59">
-        <v>8</v>
-      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -1659,9 +1635,6 @@
       <c r="D60" t="s">
         <v>73</v>
       </c>
-      <c r="E60">
-        <v>9</v>
-      </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
@@ -1675,9 +1648,6 @@
       </c>
       <c r="D61" t="s">
         <v>74</v>
-      </c>
-      <c r="E61">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cheese snacks through toilet paper posts
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE713E3-B397-46E3-B014-CFEED9A97C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6940BA23-4537-4256-BD78-5C9A744E203B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="76">
   <si>
     <t>option</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>Walk or Stroll</t>
+  </si>
+  <si>
+    <t>series_no</t>
   </si>
 </sst>
 </file>
@@ -633,1020 +636,1204 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1">
+      <c r="C2" s="1">
         <v>45992</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1">
+      <c r="C3" s="1">
         <v>45992</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="1">
+      <c r="C4" s="1">
         <v>45999</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>10</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="1">
+      <c r="C5" s="1">
         <v>45999</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1">
+      <c r="C6" s="1">
         <v>46006</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>21</v>
       </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="1">
+      <c r="C7" s="1">
         <v>46006</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1">
+      <c r="C8" s="1">
         <v>46006</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>23</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="1">
+      <c r="C9" s="1">
         <v>46006</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>3</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>24</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1">
+      <c r="C10" s="1">
         <v>46013</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>4</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>17</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="1">
+      <c r="C11" s="1">
         <v>46013</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>4</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>18</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="1">
+      <c r="C12" s="1">
         <v>46027</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>5</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>25</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="1">
+      <c r="C13" s="1">
         <v>46027</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>5</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>26</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1">
+      <c r="C14" s="1">
         <v>46034</v>
       </c>
-      <c r="C14">
-        <v>6</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="D14">
+        <v>6</v>
+      </c>
+      <c r="E14" t="s">
         <v>27</v>
       </c>
-      <c r="E14">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="F14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="1">
+      <c r="C15" s="1">
         <v>46034</v>
       </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
         <v>28</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="1">
+      <c r="C16" s="1">
         <v>46042</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>7</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>29</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="1">
+      <c r="C17" s="1">
         <v>46042</v>
       </c>
-      <c r="C17">
+      <c r="D17">
         <v>7</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>30</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
         <v>3</v>
       </c>
-      <c r="B18" s="1">
+      <c r="C18" s="1">
         <v>46042</v>
       </c>
-      <c r="C18">
-        <v>8</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="D18">
+        <v>8</v>
+      </c>
+      <c r="E18" t="s">
         <v>31</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="1">
+      <c r="C19" s="1">
         <v>46042</v>
       </c>
-      <c r="C19">
-        <v>8</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="D19">
+        <v>8</v>
+      </c>
+      <c r="E19" t="s">
         <v>32</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="1">
+      <c r="C20" s="1">
         <v>46042</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <v>9</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>33</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
         <v>3</v>
       </c>
-      <c r="B21" s="1">
+      <c r="C21" s="1">
         <v>46042</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <v>9</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>34</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
         <v>3</v>
       </c>
-      <c r="B22" s="1">
+      <c r="C22" s="1">
         <v>46042</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <v>10</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>35</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="1">
+      <c r="C23" s="1">
         <v>46042</v>
       </c>
-      <c r="C23">
+      <c r="D23">
         <v>10</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>36</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="1">
+      <c r="C24" s="1">
         <v>46063</v>
       </c>
-      <c r="C24">
+      <c r="D24">
         <v>11</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>37</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
         <v>4</v>
       </c>
-      <c r="B25" s="1">
+      <c r="C25" s="1">
         <v>46063</v>
       </c>
-      <c r="C25">
+      <c r="D25">
         <v>11</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>38</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
         <v>4</v>
       </c>
-      <c r="B26" s="1">
+      <c r="C26" s="1">
         <v>46063</v>
       </c>
-      <c r="C26">
+      <c r="D26">
         <v>12</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>39</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="1">
+      <c r="C27" s="1">
         <v>46063</v>
       </c>
-      <c r="C27">
+      <c r="D27">
         <v>12</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>40</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="1">
+      <c r="C28" s="1">
         <v>46063</v>
       </c>
-      <c r="C28">
+      <c r="D28">
         <v>13</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>41</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="1">
+      <c r="C29" s="1">
         <v>46063</v>
       </c>
-      <c r="C29">
+      <c r="D29">
         <v>13</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>42</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="1">
+      <c r="C30" s="1">
         <v>46063</v>
       </c>
-      <c r="C30">
+      <c r="D30">
         <v>14</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>43</v>
       </c>
-      <c r="E30">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="F30">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="1">
+      <c r="C31" s="1">
         <v>46063</v>
       </c>
-      <c r="C31">
+      <c r="D31">
         <v>14</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>44</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>8</v>
+      </c>
+      <c r="B32" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="1">
+      <c r="C32" s="1">
         <v>46076</v>
       </c>
-      <c r="C32">
+      <c r="D32">
         <v>15</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>45</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
         <v>5</v>
       </c>
-      <c r="B33" s="1">
+      <c r="C33" s="1">
         <v>46076</v>
       </c>
-      <c r="C33">
+      <c r="D33">
         <v>15</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>46</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>8</v>
+      </c>
+      <c r="B34" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="1">
+      <c r="C34" s="1">
         <v>46076</v>
       </c>
-      <c r="C34">
+      <c r="D34">
         <v>16</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>47</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>8</v>
+      </c>
+      <c r="B35" t="s">
         <v>5</v>
       </c>
-      <c r="B35" s="1">
+      <c r="C35" s="1">
         <v>46076</v>
       </c>
-      <c r="C35">
+      <c r="D35">
         <v>16</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>48</v>
       </c>
-      <c r="E35">
+      <c r="F35">
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>8</v>
+      </c>
+      <c r="B36" t="s">
         <v>5</v>
       </c>
-      <c r="B36" s="1">
+      <c r="C36" s="1">
         <v>46076</v>
       </c>
-      <c r="C36">
+      <c r="D36">
         <v>17</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>49</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>8</v>
+      </c>
+      <c r="B37" t="s">
         <v>5</v>
       </c>
-      <c r="B37" s="1">
+      <c r="C37" s="1">
         <v>46076</v>
       </c>
-      <c r="C37">
+      <c r="D37">
         <v>17</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>50</v>
       </c>
-      <c r="E37">
+      <c r="F37">
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>8</v>
+      </c>
+      <c r="B38" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="1">
+      <c r="C38" s="1">
         <v>46076</v>
       </c>
-      <c r="C38">
+      <c r="D38">
         <v>18</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>51</v>
       </c>
-      <c r="E38">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="F38">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>8</v>
+      </c>
+      <c r="B39" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="1">
+      <c r="C39" s="1">
         <v>46076</v>
       </c>
-      <c r="C39">
+      <c r="D39">
         <v>18</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>52</v>
       </c>
-      <c r="E39">
+      <c r="F39">
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>8</v>
+      </c>
+      <c r="B40" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="1">
+      <c r="C40" s="1">
         <v>46076</v>
       </c>
-      <c r="C40">
+      <c r="D40">
         <v>19</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40" t="s">
         <v>54</v>
       </c>
-      <c r="E40">
+      <c r="F40">
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>8</v>
+      </c>
+      <c r="B41" t="s">
         <v>5</v>
       </c>
-      <c r="B41" s="1">
+      <c r="C41" s="1">
         <v>46076</v>
       </c>
-      <c r="C41">
+      <c r="D41">
         <v>19</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
         <v>53</v>
       </c>
-      <c r="E41">
+      <c r="F41">
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>6</v>
-      </c>
-      <c r="B42" s="1">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="1">
         <v>46087</v>
       </c>
-      <c r="C42">
+      <c r="D42">
         <v>20</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>55</v>
       </c>
-      <c r="E42">
+      <c r="F42">
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>6</v>
-      </c>
-      <c r="B43" s="1">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>9</v>
+      </c>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" s="1">
         <v>46087</v>
       </c>
-      <c r="C43">
+      <c r="D43">
         <v>20</v>
       </c>
-      <c r="D43" t="s">
+      <c r="E43" t="s">
         <v>56</v>
       </c>
-      <c r="E43">
+      <c r="F43">
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>6</v>
-      </c>
-      <c r="B44" s="1">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>9</v>
+      </c>
+      <c r="B44" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="1">
         <v>46087</v>
       </c>
-      <c r="C44">
+      <c r="D44">
         <v>21</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>57</v>
       </c>
-      <c r="E44">
+      <c r="F44">
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>6</v>
-      </c>
-      <c r="B45" s="1">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>9</v>
+      </c>
+      <c r="B45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="1">
         <v>46087</v>
       </c>
-      <c r="C45">
+      <c r="D45">
         <v>21</v>
       </c>
-      <c r="D45" t="s">
+      <c r="E45" t="s">
         <v>58</v>
       </c>
-      <c r="E45">
+      <c r="F45">
         <v>20</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>6</v>
-      </c>
-      <c r="B46" s="1">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>9</v>
+      </c>
+      <c r="B46" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" s="1">
         <v>46087</v>
       </c>
-      <c r="C46">
+      <c r="D46">
         <v>22</v>
       </c>
-      <c r="D46" t="s">
+      <c r="E46" t="s">
         <v>59</v>
       </c>
-      <c r="E46">
+      <c r="F46">
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47" s="1">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>9</v>
+      </c>
+      <c r="B47" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="1">
         <v>46087</v>
       </c>
-      <c r="C47">
+      <c r="D47">
         <v>22</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>60</v>
       </c>
-      <c r="E47">
+      <c r="F47">
         <v>20</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>6</v>
-      </c>
-      <c r="B48" s="1">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>9</v>
+      </c>
+      <c r="B48" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" s="1">
         <v>46087</v>
       </c>
-      <c r="C48">
+      <c r="D48">
         <v>23</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>61</v>
       </c>
-      <c r="E48">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" s="1">
+      <c r="F48">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>9</v>
+      </c>
+      <c r="B49" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="1">
         <v>46087</v>
       </c>
-      <c r="C49">
+      <c r="D49">
         <v>23</v>
       </c>
-      <c r="D49" t="s">
+      <c r="E49" t="s">
         <v>62</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>6</v>
-      </c>
-      <c r="B50" s="1">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>9</v>
+      </c>
+      <c r="B50" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" s="1">
         <v>46087</v>
       </c>
-      <c r="C50">
+      <c r="D50">
         <v>24</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>63</v>
       </c>
-      <c r="E50">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>6</v>
-      </c>
-      <c r="B51" s="1">
+      <c r="F50">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>9</v>
+      </c>
+      <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="1">
         <v>46087</v>
       </c>
-      <c r="C51">
+      <c r="D51">
         <v>24</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>64</v>
       </c>
-      <c r="E51">
+      <c r="F51">
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>8</v>
-      </c>
-      <c r="B52" s="1">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>10</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" s="1">
         <v>46099</v>
       </c>
-      <c r="C52">
+      <c r="D52">
         <v>25</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>8</v>
-      </c>
-      <c r="B53" s="1">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" s="1">
         <v>46099</v>
       </c>
-      <c r="C53">
+      <c r="D53">
         <v>25</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>8</v>
-      </c>
-      <c r="B54" s="1">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>10</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" s="1">
         <v>46099</v>
       </c>
-      <c r="C54">
+      <c r="D54">
         <v>26</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>8</v>
-      </c>
-      <c r="B55" s="1">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>10</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" s="1">
         <v>46099</v>
       </c>
-      <c r="C55">
+      <c r="D55">
         <v>26</v>
       </c>
-      <c r="D55" t="s">
+      <c r="E55" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>8</v>
-      </c>
-      <c r="B56" s="1">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>10</v>
+      </c>
+      <c r="B56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" s="1">
         <v>46099</v>
       </c>
-      <c r="C56">
+      <c r="D56">
         <v>27</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>8</v>
-      </c>
-      <c r="B57" s="1">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>10</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" s="1">
         <v>46099</v>
       </c>
-      <c r="C57">
+      <c r="D57">
         <v>27</v>
       </c>
-      <c r="D57" t="s">
+      <c r="E57" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>8</v>
-      </c>
-      <c r="B58" s="1">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>10</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" s="1">
         <v>46099</v>
       </c>
-      <c r="C58">
+      <c r="D58">
         <v>28</v>
       </c>
-      <c r="D58" t="s">
+      <c r="E58" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>8</v>
-      </c>
-      <c r="B59" s="1">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>10</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="1">
         <v>46099</v>
       </c>
-      <c r="C59">
+      <c r="D59">
         <v>28</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>8</v>
-      </c>
-      <c r="B60" s="1">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>10</v>
+      </c>
+      <c r="B60" t="s">
+        <v>8</v>
+      </c>
+      <c r="C60" s="1">
         <v>46099</v>
       </c>
-      <c r="C60">
+      <c r="D60">
         <v>29</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>8</v>
-      </c>
-      <c r="B61" s="1">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>10</v>
+      </c>
+      <c r="B61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" s="1">
         <v>46099</v>
       </c>
-      <c r="C61">
+      <c r="D61">
         <v>29</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>74</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data updates through 6 8 2026
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03FBB8E6-1824-47D0-812C-003135551845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D82D16-9EF8-483E-905F-37852E37AD92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="11424" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,35 +36,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="201">
   <si>
     <t>option</t>
   </si>
   <si>
-    <t>votes</t>
-  </si>
-  <si>
     <t>series</t>
   </si>
   <si>
-    <t>vacation</t>
-  </si>
-  <si>
-    <t>home vibe</t>
-  </si>
-  <si>
-    <t>eggs</t>
-  </si>
-  <si>
-    <t>commute</t>
-  </si>
-  <si>
     <t>week</t>
   </si>
   <si>
-    <t>cherry blossoms</t>
-  </si>
-  <si>
     <t>question</t>
   </si>
   <si>
@@ -86,9 +68,6 @@
     <t>toilet paper</t>
   </si>
   <si>
-    <t>breakfast foods</t>
-  </si>
-  <si>
     <t>Over</t>
   </si>
   <si>
@@ -264,6 +243,402 @@
   </si>
   <si>
     <t>series_no</t>
+  </si>
+  <si>
+    <t>Pulp</t>
+  </si>
+  <si>
+    <t>No Pulp</t>
+  </si>
+  <si>
+    <t>Orange Juice</t>
+  </si>
+  <si>
+    <t>Donuts</t>
+  </si>
+  <si>
+    <t>Pizza Style</t>
+  </si>
+  <si>
+    <t>Mac &amp; Cheese</t>
+  </si>
+  <si>
+    <t>Peanut Butter</t>
+  </si>
+  <si>
+    <t>Chocolate Chip Cookies</t>
+  </si>
+  <si>
+    <t>Pickles</t>
+  </si>
+  <si>
+    <t>Yeasted</t>
+  </si>
+  <si>
+    <t>Cakey</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Square</t>
+  </si>
+  <si>
+    <t>Creamy Stovetop</t>
+  </si>
+  <si>
+    <t>Baked w/ Crust</t>
+  </si>
+  <si>
+    <t>Creamy</t>
+  </si>
+  <si>
+    <t>Chunky</t>
+  </si>
+  <si>
+    <t>Soft &amp; Chewy</t>
+  </si>
+  <si>
+    <t>Thin &amp; Crispy</t>
+  </si>
+  <si>
+    <t>Dill</t>
+  </si>
+  <si>
+    <t>Bread &amp; Butter</t>
+  </si>
+  <si>
+    <t>hq_votes</t>
+  </si>
+  <si>
+    <t>rtp_votes</t>
+  </si>
+  <si>
+    <t>soft stack</t>
+  </si>
+  <si>
+    <t>flavor profile</t>
+  </si>
+  <si>
+    <t>Climate</t>
+  </si>
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Style</t>
+  </si>
+  <si>
+    <t>Destination</t>
+  </si>
+  <si>
+    <t>Décor</t>
+  </si>
+  <si>
+    <t>Vibe</t>
+  </si>
+  <si>
+    <t>Atmosphere</t>
+  </si>
+  <si>
+    <t>Utility</t>
+  </si>
+  <si>
+    <t>In a pan</t>
+  </si>
+  <si>
+    <t>In a pot</t>
+  </si>
+  <si>
+    <t>Yolk</t>
+  </si>
+  <si>
+    <t>Condiment</t>
+  </si>
+  <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>Audio</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>Biking</t>
+  </si>
+  <si>
+    <t>Escalators</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Enjoying Nature</t>
+  </si>
+  <si>
+    <t>Swimming</t>
+  </si>
+  <si>
+    <t>Animal Scoping</t>
+  </si>
+  <si>
+    <t>Volunteering</t>
+  </si>
+  <si>
+    <t>Hike</t>
+  </si>
+  <si>
+    <t>Lake</t>
+  </si>
+  <si>
+    <t>Ocean</t>
+  </si>
+  <si>
+    <t>Birding</t>
+  </si>
+  <si>
+    <t>Snorkling</t>
+  </si>
+  <si>
+    <t>Trash Pickup</t>
+  </si>
+  <si>
+    <t>Invasive Species Removal</t>
+  </si>
+  <si>
+    <t>Spiky</t>
+  </si>
+  <si>
+    <t>Hedgehog</t>
+  </si>
+  <si>
+    <t>Porcupine</t>
+  </si>
+  <si>
+    <t>Pinnipeds</t>
+  </si>
+  <si>
+    <t>Seal</t>
+  </si>
+  <si>
+    <t>Sea Lion</t>
+  </si>
+  <si>
+    <t>Insect-Eaters</t>
+  </si>
+  <si>
+    <t>Armadillo</t>
+  </si>
+  <si>
+    <t>Pangolin</t>
+  </si>
+  <si>
+    <t>Crocodylia</t>
+  </si>
+  <si>
+    <t>Corvidae</t>
+  </si>
+  <si>
+    <t>Alligator</t>
+  </si>
+  <si>
+    <t>Crocodile</t>
+  </si>
+  <si>
+    <t>Raven</t>
+  </si>
+  <si>
+    <t>Crow</t>
+  </si>
+  <si>
+    <t>Lepidoptera</t>
+  </si>
+  <si>
+    <t>Anura</t>
+  </si>
+  <si>
+    <t>Moth</t>
+  </si>
+  <si>
+    <t>Butterfly</t>
+  </si>
+  <si>
+    <t>Frog</t>
+  </si>
+  <si>
+    <t>Toad</t>
+  </si>
+  <si>
+    <t>Sandwich</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>complete</t>
+  </si>
+  <si>
+    <t>polling</t>
+  </si>
+  <si>
+    <t>Cheese Snacks</t>
+  </si>
+  <si>
+    <t>Cats vs. Dogs</t>
+  </si>
+  <si>
+    <t>Holiday Drinks</t>
+  </si>
+  <si>
+    <t>Toilet Paper</t>
+  </si>
+  <si>
+    <t>Breakfast Foods</t>
+  </si>
+  <si>
+    <t>Vacation</t>
+  </si>
+  <si>
+    <t>Home Vibe</t>
+  </si>
+  <si>
+    <t>Eggs</t>
+  </si>
+  <si>
+    <t>Commute</t>
+  </si>
+  <si>
+    <t>Cherry Blossoms</t>
+  </si>
+  <si>
+    <t>Food Face-Offs</t>
+  </si>
+  <si>
+    <t>Earth Day</t>
+  </si>
+  <si>
+    <t>Animal Match-Ups</t>
+  </si>
+  <si>
+    <t>NBA Finals</t>
+  </si>
+  <si>
+    <t>Dessert Match-Ups Part I</t>
+  </si>
+  <si>
+    <t>Fruity</t>
+  </si>
+  <si>
+    <t>Cobbler</t>
+  </si>
+  <si>
+    <t>Pie</t>
+  </si>
+  <si>
+    <t>Mousse</t>
+  </si>
+  <si>
+    <t>Pudding</t>
+  </si>
+  <si>
+    <t>Tiramisu</t>
+  </si>
+  <si>
+    <t>Crème Brulee</t>
+  </si>
+  <si>
+    <t>Ice Cream</t>
+  </si>
+  <si>
+    <t>Frozen Yogurt</t>
+  </si>
+  <si>
+    <t>Cannoli</t>
+  </si>
+  <si>
+    <t>Éclair</t>
+  </si>
+  <si>
+    <t>Layered</t>
+  </si>
+  <si>
+    <t>Frozen</t>
+  </si>
+  <si>
+    <t>Stuffed</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Breakfast</t>
+  </si>
+  <si>
+    <t>Meats</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>Seasons</t>
+  </si>
+  <si>
+    <t>Grocery</t>
+  </si>
+  <si>
+    <t>Catchphrase</t>
+  </si>
+  <si>
+    <t>Knicks</t>
+  </si>
+  <si>
+    <t>Spurs</t>
+  </si>
+  <si>
+    <t>Bagel Sandwich</t>
+  </si>
+  <si>
+    <t>Breakfast Taco</t>
+  </si>
+  <si>
+    <t>Hot Pastrami</t>
+  </si>
+  <si>
+    <t>Smoked Brisket</t>
+  </si>
+  <si>
+    <t>Subway</t>
+  </si>
+  <si>
+    <t>Pickup Truck</t>
+  </si>
+  <si>
+    <t>Four Seasons</t>
+  </si>
+  <si>
+    <t>Mild Winter</t>
+  </si>
+  <si>
+    <t>Bodega</t>
+  </si>
+  <si>
+    <t>HEB</t>
+  </si>
+  <si>
+    <t>"I'm walkin' here"</t>
+  </si>
+  <si>
+    <t>"Bless your heart"</t>
   </si>
 </sst>
 </file>
@@ -636,1235 +1011,2826 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+      <c r="G1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="C2" s="1">
         <v>45992</v>
       </c>
-      <c r="D2">
-        <v>1</v>
+      <c r="D2" t="s">
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F2">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="C3" s="1">
         <v>45992</v>
       </c>
-      <c r="D3">
-        <v>1</v>
+      <c r="D3" t="s">
+        <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F3">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="C4" s="1">
         <v>45999</v>
       </c>
-      <c r="D4">
-        <v>2</v>
+      <c r="D4" t="s">
+        <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F4">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="C5" s="1">
         <v>45999</v>
       </c>
-      <c r="D5">
-        <v>2</v>
+      <c r="D5" t="s">
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F5">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="C6" s="1">
         <v>46006</v>
       </c>
-      <c r="D6">
-        <v>3</v>
+      <c r="D6" t="s">
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F6">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="C7" s="1">
         <v>46006</v>
       </c>
-      <c r="D7">
-        <v>3</v>
+      <c r="D7" t="s">
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F7">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H7" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="C8" s="1">
         <v>46006</v>
       </c>
-      <c r="D8">
-        <v>3</v>
+      <c r="D8" t="s">
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F8">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="C9" s="1">
         <v>46006</v>
       </c>
-      <c r="D9">
-        <v>3</v>
+      <c r="D9" t="s">
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F9">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="C10" s="1">
         <v>46013</v>
       </c>
-      <c r="D10">
-        <v>4</v>
+      <c r="D10" t="s">
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F10">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="C11" s="1">
         <v>46013</v>
       </c>
-      <c r="D11">
-        <v>4</v>
+      <c r="D11" t="s">
+        <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F11">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="C12" s="1">
         <v>46027</v>
       </c>
-      <c r="D12">
-        <v>5</v>
+      <c r="D12" t="s">
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F12">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="C13" s="1">
         <v>46027</v>
       </c>
-      <c r="D13">
-        <v>5</v>
+      <c r="D13" t="s">
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="F13">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="C14" s="1">
         <v>46034</v>
       </c>
-      <c r="D14">
-        <v>6</v>
+      <c r="D14" t="s">
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F14">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H14" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="C15" s="1">
         <v>46034</v>
       </c>
-      <c r="D15">
-        <v>6</v>
+      <c r="D15" t="s">
+        <v>93</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F15">
         <v>13</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C16" s="1">
         <v>46042</v>
       </c>
-      <c r="D16">
-        <v>7</v>
+      <c r="D16" t="s">
+        <v>94</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F16">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C17" s="1">
         <v>46042</v>
       </c>
-      <c r="D17">
-        <v>7</v>
+      <c r="D17" t="s">
+        <v>94</v>
       </c>
       <c r="E17" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F17">
         <v>9</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C18" s="1">
         <v>46042</v>
       </c>
-      <c r="D18">
-        <v>8</v>
+      <c r="D18" t="s">
+        <v>95</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="F18">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C19" s="1">
         <v>46042</v>
       </c>
-      <c r="D19">
-        <v>8</v>
+      <c r="D19" t="s">
+        <v>95</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="F19">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C20" s="1">
         <v>46042</v>
       </c>
-      <c r="D20">
-        <v>9</v>
+      <c r="D20" t="s">
+        <v>96</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F20">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C21" s="1">
         <v>46042</v>
       </c>
-      <c r="D21">
-        <v>9</v>
+      <c r="D21" t="s">
+        <v>96</v>
       </c>
       <c r="E21" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="F21">
         <v>23</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H21" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C22" s="1">
         <v>46042</v>
       </c>
-      <c r="D22">
-        <v>10</v>
+      <c r="D22" t="s">
+        <v>97</v>
       </c>
       <c r="E22" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F22">
         <v>24</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>3</v>
+        <v>156</v>
       </c>
       <c r="C23" s="1">
         <v>46042</v>
       </c>
-      <c r="D23">
-        <v>10</v>
+      <c r="D23" t="s">
+        <v>97</v>
       </c>
       <c r="E23" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F23">
         <v>9</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C24" s="1">
         <v>46063</v>
       </c>
-      <c r="D24">
-        <v>11</v>
+      <c r="D24" t="s">
+        <v>101</v>
       </c>
       <c r="E24" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F24">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H24" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C25" s="1">
         <v>46063</v>
       </c>
-      <c r="D25">
-        <v>11</v>
+      <c r="D25" t="s">
+        <v>101</v>
       </c>
       <c r="E25" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F25">
         <v>18</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C26" s="1">
         <v>46063</v>
       </c>
-      <c r="D26">
-        <v>12</v>
+      <c r="D26" t="s">
+        <v>99</v>
       </c>
       <c r="E26" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="F26">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C27" s="1">
         <v>46063</v>
       </c>
-      <c r="D27">
-        <v>12</v>
+      <c r="D27" t="s">
+        <v>99</v>
       </c>
       <c r="E27" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F27">
         <v>7</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C28" s="1">
         <v>46063</v>
       </c>
-      <c r="D28">
-        <v>13</v>
+      <c r="D28" t="s">
+        <v>100</v>
       </c>
       <c r="E28" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F28">
         <v>18</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H28" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>7</v>
       </c>
       <c r="B29" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C29" s="1">
         <v>46063</v>
       </c>
-      <c r="D29">
-        <v>13</v>
+      <c r="D29" t="s">
+        <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F29">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C30" s="1">
         <v>46063</v>
       </c>
-      <c r="D30">
-        <v>14</v>
+      <c r="D30" t="s">
+        <v>98</v>
       </c>
       <c r="E30" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F30">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H30" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>7</v>
       </c>
       <c r="B31" t="s">
-        <v>4</v>
+        <v>157</v>
       </c>
       <c r="C31" s="1">
         <v>46063</v>
       </c>
-      <c r="D31">
-        <v>14</v>
+      <c r="D31" t="s">
+        <v>98</v>
       </c>
       <c r="E31" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F31">
         <v>20</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C32" s="1">
         <v>46076</v>
       </c>
-      <c r="D32">
-        <v>15</v>
+      <c r="D32" t="s">
+        <v>102</v>
       </c>
       <c r="E32" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F32">
         <v>11</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H32" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C33" s="1">
         <v>46076</v>
       </c>
-      <c r="D33">
-        <v>15</v>
+      <c r="D33" t="s">
+        <v>102</v>
       </c>
       <c r="E33" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="F33">
         <v>20</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H33" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C34" s="1">
         <v>46076</v>
       </c>
-      <c r="D34">
-        <v>16</v>
+      <c r="D34" t="s">
+        <v>103</v>
       </c>
       <c r="E34" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F34">
         <v>13</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H34" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C35" s="1">
         <v>46076</v>
       </c>
-      <c r="D35">
-        <v>16</v>
+      <c r="D35" t="s">
+        <v>103</v>
       </c>
       <c r="E35" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F35">
         <v>13</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C36" s="1">
         <v>46076</v>
       </c>
-      <c r="D36">
-        <v>17</v>
+      <c r="D36" t="s">
+        <v>104</v>
       </c>
       <c r="E36" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F36">
         <v>17</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H36" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C37" s="1">
         <v>46076</v>
       </c>
-      <c r="D37">
-        <v>17</v>
+      <c r="D37" t="s">
+        <v>104</v>
       </c>
       <c r="E37" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F37">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H37" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C38" s="1">
         <v>46076</v>
       </c>
-      <c r="D38">
-        <v>18</v>
+      <c r="D38" t="s">
+        <v>105</v>
       </c>
       <c r="E38" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F38">
         <v>6</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H38" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C39" s="1">
         <v>46076</v>
       </c>
-      <c r="D39">
-        <v>18</v>
+      <c r="D39" t="s">
+        <v>105</v>
       </c>
       <c r="E39" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="F39">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H39" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C40" s="1">
         <v>46076</v>
       </c>
-      <c r="D40">
-        <v>19</v>
+      <c r="D40" t="s">
+        <v>147</v>
       </c>
       <c r="E40" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F40">
         <v>18</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H40" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C41" s="1">
         <v>46076</v>
       </c>
-      <c r="D41">
-        <v>19</v>
+      <c r="D41" t="s">
+        <v>147</v>
       </c>
       <c r="E41" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F41">
         <v>4</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H41" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C42" s="1">
         <v>46087</v>
       </c>
-      <c r="D42">
-        <v>20</v>
+      <c r="D42" t="s">
+        <v>106</v>
       </c>
       <c r="E42" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="F42">
         <v>23</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H42" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C43" s="1">
         <v>46087</v>
       </c>
-      <c r="D43">
-        <v>20</v>
+      <c r="D43" t="s">
+        <v>106</v>
       </c>
       <c r="E43" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="F43">
         <v>15</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H43" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>9</v>
       </c>
       <c r="B44" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C44" s="1">
         <v>46087</v>
       </c>
-      <c r="D44">
-        <v>21</v>
+      <c r="D44" t="s">
+        <v>107</v>
       </c>
       <c r="E44" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F44">
         <v>21</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H44" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>9</v>
       </c>
       <c r="B45" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C45" s="1">
         <v>46087</v>
       </c>
-      <c r="D45">
-        <v>21</v>
+      <c r="D45" t="s">
+        <v>107</v>
       </c>
       <c r="E45" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="F45">
         <v>20</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H45" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
       <c r="B46" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C46" s="1">
         <v>46087</v>
       </c>
-      <c r="D46">
-        <v>22</v>
+      <c r="D46" t="s">
+        <v>108</v>
       </c>
       <c r="E46" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="F46">
         <v>10</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H46" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>9</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C47" s="1">
         <v>46087</v>
       </c>
-      <c r="D47">
-        <v>22</v>
+      <c r="D47" t="s">
+        <v>108</v>
       </c>
       <c r="E47" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F47">
         <v>20</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>9</v>
       </c>
       <c r="B48" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C48" s="1">
         <v>46087</v>
       </c>
-      <c r="D48">
-        <v>23</v>
+      <c r="D48" t="s">
+        <v>109</v>
       </c>
       <c r="E48" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F48">
         <v>6</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H48" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>9</v>
       </c>
       <c r="B49" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C49" s="1">
         <v>46087</v>
       </c>
-      <c r="D49">
-        <v>23</v>
+      <c r="D49" t="s">
+        <v>109</v>
       </c>
       <c r="E49" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F49">
         <v>14</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H49" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>9</v>
       </c>
       <c r="B50" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C50" s="1">
         <v>46087</v>
       </c>
-      <c r="D50">
-        <v>24</v>
+      <c r="D50" t="s">
+        <v>110</v>
       </c>
       <c r="E50" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F50">
         <v>6</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H50" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>6</v>
+        <v>159</v>
       </c>
       <c r="C51" s="1">
         <v>46087</v>
       </c>
-      <c r="D51">
-        <v>24</v>
+      <c r="D51" t="s">
+        <v>110</v>
       </c>
       <c r="E51" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F51">
         <v>34</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H51" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C52" s="1">
         <v>46099</v>
       </c>
-      <c r="D52">
-        <v>25</v>
+      <c r="D52" t="s">
+        <v>111</v>
       </c>
       <c r="E52" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F52">
         <v>25</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H52" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C53" s="1">
         <v>46099</v>
       </c>
-      <c r="D53">
-        <v>25</v>
+      <c r="D53" t="s">
+        <v>111</v>
       </c>
       <c r="E53" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F53">
         <v>13</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H53" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C54" s="1">
         <v>46099</v>
       </c>
-      <c r="D54">
-        <v>26</v>
+      <c r="D54" t="s">
+        <v>99</v>
       </c>
       <c r="E54" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="F54">
         <v>8</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H54" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10</v>
       </c>
       <c r="B55" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C55" s="1">
         <v>46099</v>
       </c>
-      <c r="D55">
-        <v>26</v>
+      <c r="D55" t="s">
+        <v>99</v>
       </c>
       <c r="E55" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="F55">
         <v>29</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H55" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C56" s="1">
         <v>46099</v>
       </c>
-      <c r="D56">
-        <v>27</v>
+      <c r="D56" t="s">
+        <v>112</v>
       </c>
       <c r="E56" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F56">
         <v>21</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H56" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C57" s="1">
         <v>46099</v>
       </c>
-      <c r="D57">
-        <v>27</v>
+      <c r="D57" t="s">
+        <v>112</v>
       </c>
       <c r="E57" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F57">
         <v>14</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H57" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C58" s="1">
         <v>46099</v>
       </c>
-      <c r="D58">
-        <v>28</v>
+      <c r="D58" t="s">
+        <v>113</v>
       </c>
       <c r="E58" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F58">
         <v>22</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H58" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C59" s="1">
         <v>46099</v>
       </c>
-      <c r="D59">
-        <v>28</v>
+      <c r="D59" t="s">
+        <v>113</v>
       </c>
       <c r="E59" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F59">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H59" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C60" s="1">
         <v>46099</v>
       </c>
-      <c r="D60">
-        <v>29</v>
+      <c r="D60" t="s">
+        <v>114</v>
       </c>
       <c r="E60" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H60" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10</v>
       </c>
       <c r="B61" t="s">
-        <v>8</v>
+        <v>160</v>
       </c>
       <c r="C61" s="1">
         <v>46099</v>
       </c>
-      <c r="D61">
-        <v>29</v>
+      <c r="D61" t="s">
+        <v>114</v>
       </c>
       <c r="E61" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="F61">
         <v>28</v>
+      </c>
+      <c r="H61" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>11</v>
+      </c>
+      <c r="B62" t="s">
+        <v>161</v>
+      </c>
+      <c r="C62" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D62" t="s">
+        <v>71</v>
+      </c>
+      <c r="E62" t="s">
+        <v>69</v>
+      </c>
+      <c r="F62">
+        <v>27</v>
+      </c>
+      <c r="H62" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>11</v>
+      </c>
+      <c r="B63" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D63" t="s">
+        <v>71</v>
+      </c>
+      <c r="E63" t="s">
+        <v>70</v>
+      </c>
+      <c r="F63">
+        <v>22</v>
+      </c>
+      <c r="H63" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>11</v>
+      </c>
+      <c r="B64" t="s">
+        <v>161</v>
+      </c>
+      <c r="C64" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D64" t="s">
+        <v>72</v>
+      </c>
+      <c r="E64" t="s">
+        <v>78</v>
+      </c>
+      <c r="F64">
+        <v>26</v>
+      </c>
+      <c r="H64" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>11</v>
+      </c>
+      <c r="B65" t="s">
+        <v>161</v>
+      </c>
+      <c r="C65" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D65" t="s">
+        <v>72</v>
+      </c>
+      <c r="E65" t="s">
+        <v>79</v>
+      </c>
+      <c r="F65">
+        <v>19</v>
+      </c>
+      <c r="H65" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>11</v>
+      </c>
+      <c r="B66" t="s">
+        <v>161</v>
+      </c>
+      <c r="C66" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D66" t="s">
+        <v>73</v>
+      </c>
+      <c r="E66" t="s">
+        <v>80</v>
+      </c>
+      <c r="F66">
+        <v>35</v>
+      </c>
+      <c r="H66" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>11</v>
+      </c>
+      <c r="B67" t="s">
+        <v>161</v>
+      </c>
+      <c r="C67" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D67" t="s">
+        <v>73</v>
+      </c>
+      <c r="E67" t="s">
+        <v>81</v>
+      </c>
+      <c r="F67">
+        <v>10</v>
+      </c>
+      <c r="H67" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>11</v>
+      </c>
+      <c r="B68" t="s">
+        <v>161</v>
+      </c>
+      <c r="C68" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D68" t="s">
+        <v>74</v>
+      </c>
+      <c r="E68" t="s">
+        <v>82</v>
+      </c>
+      <c r="F68">
+        <v>20</v>
+      </c>
+      <c r="H68" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>11</v>
+      </c>
+      <c r="B69" t="s">
+        <v>161</v>
+      </c>
+      <c r="C69" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D69" t="s">
+        <v>74</v>
+      </c>
+      <c r="E69" t="s">
+        <v>83</v>
+      </c>
+      <c r="F69">
+        <v>28</v>
+      </c>
+      <c r="H69" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>11</v>
+      </c>
+      <c r="B70" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D70" t="s">
+        <v>75</v>
+      </c>
+      <c r="E70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F70">
+        <v>28</v>
+      </c>
+      <c r="H70" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>11</v>
+      </c>
+      <c r="B71" t="s">
+        <v>161</v>
+      </c>
+      <c r="C71" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D71" t="s">
+        <v>75</v>
+      </c>
+      <c r="E71" t="s">
+        <v>85</v>
+      </c>
+      <c r="F71">
+        <v>21</v>
+      </c>
+      <c r="H71" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>11</v>
+      </c>
+      <c r="B72" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D72" t="s">
+        <v>76</v>
+      </c>
+      <c r="E72" t="s">
+        <v>86</v>
+      </c>
+      <c r="F72">
+        <v>32</v>
+      </c>
+      <c r="H72" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>11</v>
+      </c>
+      <c r="B73" t="s">
+        <v>161</v>
+      </c>
+      <c r="C73" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D73" t="s">
+        <v>76</v>
+      </c>
+      <c r="E73" t="s">
+        <v>87</v>
+      </c>
+      <c r="F73">
+        <v>11</v>
+      </c>
+      <c r="H73" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>11</v>
+      </c>
+      <c r="B74" t="s">
+        <v>161</v>
+      </c>
+      <c r="C74" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D74" t="s">
+        <v>77</v>
+      </c>
+      <c r="E74" t="s">
+        <v>88</v>
+      </c>
+      <c r="F74">
+        <v>34</v>
+      </c>
+      <c r="H74" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>11</v>
+      </c>
+      <c r="B75" t="s">
+        <v>161</v>
+      </c>
+      <c r="C75" s="1">
+        <v>46125</v>
+      </c>
+      <c r="D75" t="s">
+        <v>77</v>
+      </c>
+      <c r="E75" t="s">
+        <v>89</v>
+      </c>
+      <c r="F75">
+        <v>9</v>
+      </c>
+      <c r="H75" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>12</v>
+      </c>
+      <c r="B76" t="s">
+        <v>162</v>
+      </c>
+      <c r="C76" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D76" t="s">
+        <v>115</v>
+      </c>
+      <c r="E76" t="s">
+        <v>66</v>
+      </c>
+      <c r="F76">
+        <v>7</v>
+      </c>
+      <c r="G76">
+        <v>6</v>
+      </c>
+      <c r="H76" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>12</v>
+      </c>
+      <c r="B77" t="s">
+        <v>162</v>
+      </c>
+      <c r="C77" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D77" t="s">
+        <v>115</v>
+      </c>
+      <c r="E77" t="s">
+        <v>119</v>
+      </c>
+      <c r="F77">
+        <v>32</v>
+      </c>
+      <c r="G77">
+        <v>27</v>
+      </c>
+      <c r="H77" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>12</v>
+      </c>
+      <c r="B78" t="s">
+        <v>162</v>
+      </c>
+      <c r="C78" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D78" t="s">
+        <v>116</v>
+      </c>
+      <c r="E78" t="s">
+        <v>120</v>
+      </c>
+      <c r="F78">
+        <v>19</v>
+      </c>
+      <c r="G78">
+        <v>12</v>
+      </c>
+      <c r="H78" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>12</v>
+      </c>
+      <c r="B79" t="s">
+        <v>162</v>
+      </c>
+      <c r="C79" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D79" t="s">
+        <v>116</v>
+      </c>
+      <c r="E79" t="s">
+        <v>121</v>
+      </c>
+      <c r="F79">
+        <v>25</v>
+      </c>
+      <c r="G79">
+        <v>21</v>
+      </c>
+      <c r="H79" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>12</v>
+      </c>
+      <c r="B80" t="s">
+        <v>162</v>
+      </c>
+      <c r="C80" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D80" t="s">
+        <v>117</v>
+      </c>
+      <c r="E80" t="s">
+        <v>122</v>
+      </c>
+      <c r="F80">
+        <v>11</v>
+      </c>
+      <c r="G80">
+        <v>12</v>
+      </c>
+      <c r="H80" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>12</v>
+      </c>
+      <c r="B81" t="s">
+        <v>162</v>
+      </c>
+      <c r="C81" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D81" t="s">
+        <v>117</v>
+      </c>
+      <c r="E81" t="s">
+        <v>123</v>
+      </c>
+      <c r="F81">
+        <v>27</v>
+      </c>
+      <c r="G81">
+        <v>23</v>
+      </c>
+      <c r="H81" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>12</v>
+      </c>
+      <c r="B82" t="s">
+        <v>162</v>
+      </c>
+      <c r="C82" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D82" t="s">
+        <v>118</v>
+      </c>
+      <c r="E82" t="s">
+        <v>124</v>
+      </c>
+      <c r="F82">
+        <v>17</v>
+      </c>
+      <c r="G82">
+        <v>20</v>
+      </c>
+      <c r="H82" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>12</v>
+      </c>
+      <c r="B83" t="s">
+        <v>162</v>
+      </c>
+      <c r="C83" s="1">
+        <v>46150</v>
+      </c>
+      <c r="D83" t="s">
+        <v>118</v>
+      </c>
+      <c r="E83" t="s">
+        <v>125</v>
+      </c>
+      <c r="F83">
+        <v>21</v>
+      </c>
+      <c r="G83">
+        <v>14</v>
+      </c>
+      <c r="H83" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>13</v>
+      </c>
+      <c r="B84" t="s">
+        <v>163</v>
+      </c>
+      <c r="C84" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D84" t="s">
+        <v>126</v>
+      </c>
+      <c r="E84" t="s">
+        <v>127</v>
+      </c>
+      <c r="F84">
+        <v>24</v>
+      </c>
+      <c r="G84">
+        <v>21</v>
+      </c>
+      <c r="H84" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>13</v>
+      </c>
+      <c r="B85" t="s">
+        <v>163</v>
+      </c>
+      <c r="C85" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D85" t="s">
+        <v>126</v>
+      </c>
+      <c r="E85" t="s">
+        <v>128</v>
+      </c>
+      <c r="F85">
+        <v>10</v>
+      </c>
+      <c r="G85">
+        <v>8</v>
+      </c>
+      <c r="H85" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>13</v>
+      </c>
+      <c r="B86" t="s">
+        <v>163</v>
+      </c>
+      <c r="C86" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D86" t="s">
+        <v>129</v>
+      </c>
+      <c r="E86" t="s">
+        <v>130</v>
+      </c>
+      <c r="F86">
+        <v>18</v>
+      </c>
+      <c r="G86">
+        <v>16</v>
+      </c>
+      <c r="H86" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>13</v>
+      </c>
+      <c r="B87" t="s">
+        <v>163</v>
+      </c>
+      <c r="C87" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D87" t="s">
+        <v>129</v>
+      </c>
+      <c r="E87" t="s">
+        <v>131</v>
+      </c>
+      <c r="F87">
+        <v>16</v>
+      </c>
+      <c r="G87">
+        <v>11</v>
+      </c>
+      <c r="H87" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>13</v>
+      </c>
+      <c r="B88" t="s">
+        <v>163</v>
+      </c>
+      <c r="C88" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D88" t="s">
+        <v>132</v>
+      </c>
+      <c r="E88" t="s">
+        <v>133</v>
+      </c>
+      <c r="F88">
+        <v>21</v>
+      </c>
+      <c r="G88">
+        <v>14</v>
+      </c>
+      <c r="H88" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>13</v>
+      </c>
+      <c r="B89" t="s">
+        <v>163</v>
+      </c>
+      <c r="C89" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D89" t="s">
+        <v>132</v>
+      </c>
+      <c r="E89" t="s">
+        <v>134</v>
+      </c>
+      <c r="F89">
+        <v>12</v>
+      </c>
+      <c r="G89">
+        <v>14</v>
+      </c>
+      <c r="H89" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>13</v>
+      </c>
+      <c r="B90" t="s">
+        <v>163</v>
+      </c>
+      <c r="C90" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D90" t="s">
+        <v>135</v>
+      </c>
+      <c r="E90" t="s">
+        <v>137</v>
+      </c>
+      <c r="F90">
+        <v>17</v>
+      </c>
+      <c r="G90">
+        <v>16</v>
+      </c>
+      <c r="H90" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>13</v>
+      </c>
+      <c r="B91" t="s">
+        <v>163</v>
+      </c>
+      <c r="C91" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D91" t="s">
+        <v>135</v>
+      </c>
+      <c r="E91" t="s">
+        <v>138</v>
+      </c>
+      <c r="F91">
+        <v>16</v>
+      </c>
+      <c r="G91">
+        <v>12</v>
+      </c>
+      <c r="H91" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>13</v>
+      </c>
+      <c r="B92" t="s">
+        <v>163</v>
+      </c>
+      <c r="C92" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D92" t="s">
+        <v>136</v>
+      </c>
+      <c r="E92" t="s">
+        <v>139</v>
+      </c>
+      <c r="F92">
+        <v>22</v>
+      </c>
+      <c r="G92">
+        <v>19</v>
+      </c>
+      <c r="H92" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>13</v>
+      </c>
+      <c r="B93" t="s">
+        <v>163</v>
+      </c>
+      <c r="C93" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D93" t="s">
+        <v>136</v>
+      </c>
+      <c r="E93" t="s">
+        <v>140</v>
+      </c>
+      <c r="F93">
+        <v>12</v>
+      </c>
+      <c r="G93">
+        <v>9</v>
+      </c>
+      <c r="H93" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>13</v>
+      </c>
+      <c r="B94" t="s">
+        <v>163</v>
+      </c>
+      <c r="C94" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D94" t="s">
+        <v>141</v>
+      </c>
+      <c r="E94" t="s">
+        <v>143</v>
+      </c>
+      <c r="F94">
+        <v>9</v>
+      </c>
+      <c r="G94">
+        <v>11</v>
+      </c>
+      <c r="H94" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>13</v>
+      </c>
+      <c r="B95" t="s">
+        <v>163</v>
+      </c>
+      <c r="C95" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D95" t="s">
+        <v>141</v>
+      </c>
+      <c r="E95" t="s">
+        <v>144</v>
+      </c>
+      <c r="F95">
+        <v>25</v>
+      </c>
+      <c r="G95">
+        <v>19</v>
+      </c>
+      <c r="H95" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>13</v>
+      </c>
+      <c r="B96" t="s">
+        <v>163</v>
+      </c>
+      <c r="C96" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D96" t="s">
+        <v>142</v>
+      </c>
+      <c r="E96" t="s">
+        <v>145</v>
+      </c>
+      <c r="F96">
+        <v>24</v>
+      </c>
+      <c r="G96">
+        <v>18</v>
+      </c>
+      <c r="H96" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>13</v>
+      </c>
+      <c r="B97" t="s">
+        <v>163</v>
+      </c>
+      <c r="C97" s="1">
+        <v>46164</v>
+      </c>
+      <c r="D97" t="s">
+        <v>142</v>
+      </c>
+      <c r="E97" t="s">
+        <v>146</v>
+      </c>
+      <c r="F97">
+        <v>10</v>
+      </c>
+      <c r="G97">
+        <v>11</v>
+      </c>
+      <c r="H97" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>14</v>
+      </c>
+      <c r="B98" t="s">
+        <v>165</v>
+      </c>
+      <c r="C98" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D98" t="s">
+        <v>166</v>
+      </c>
+      <c r="E98" t="s">
+        <v>167</v>
+      </c>
+      <c r="F98">
+        <v>19</v>
+      </c>
+      <c r="H98" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>14</v>
+      </c>
+      <c r="B99" t="s">
+        <v>165</v>
+      </c>
+      <c r="C99" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D99" t="s">
+        <v>166</v>
+      </c>
+      <c r="E99" t="s">
+        <v>168</v>
+      </c>
+      <c r="F99">
+        <v>32</v>
+      </c>
+      <c r="H99" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>14</v>
+      </c>
+      <c r="B100" t="s">
+        <v>165</v>
+      </c>
+      <c r="C100" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D100" t="s">
+        <v>84</v>
+      </c>
+      <c r="E100" t="s">
+        <v>169</v>
+      </c>
+      <c r="F100">
+        <v>28</v>
+      </c>
+      <c r="H100" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>14</v>
+      </c>
+      <c r="B101" t="s">
+        <v>165</v>
+      </c>
+      <c r="C101" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D101" t="s">
+        <v>84</v>
+      </c>
+      <c r="E101" t="s">
+        <v>170</v>
+      </c>
+      <c r="F101">
+        <v>22</v>
+      </c>
+      <c r="H101" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>14</v>
+      </c>
+      <c r="B102" t="s">
+        <v>165</v>
+      </c>
+      <c r="C102" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D102" t="s">
+        <v>177</v>
+      </c>
+      <c r="E102" t="s">
+        <v>171</v>
+      </c>
+      <c r="F102">
+        <v>25</v>
+      </c>
+      <c r="H102" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103">
+        <v>14</v>
+      </c>
+      <c r="B103" t="s">
+        <v>165</v>
+      </c>
+      <c r="C103" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D103" t="s">
+        <v>177</v>
+      </c>
+      <c r="E103" t="s">
+        <v>172</v>
+      </c>
+      <c r="F103">
+        <v>27</v>
+      </c>
+      <c r="H103" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>14</v>
+      </c>
+      <c r="B104" t="s">
+        <v>165</v>
+      </c>
+      <c r="C104" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D104" t="s">
+        <v>178</v>
+      </c>
+      <c r="E104" t="s">
+        <v>173</v>
+      </c>
+      <c r="F104">
+        <v>44</v>
+      </c>
+      <c r="H104" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105">
+        <v>14</v>
+      </c>
+      <c r="B105" t="s">
+        <v>165</v>
+      </c>
+      <c r="C105" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D105" t="s">
+        <v>178</v>
+      </c>
+      <c r="E105" t="s">
+        <v>174</v>
+      </c>
+      <c r="F105">
+        <v>9</v>
+      </c>
+      <c r="H105" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106">
+        <v>14</v>
+      </c>
+      <c r="B106" t="s">
+        <v>165</v>
+      </c>
+      <c r="C106" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D106" t="s">
+        <v>179</v>
+      </c>
+      <c r="E106" t="s">
+        <v>175</v>
+      </c>
+      <c r="F106">
+        <v>30</v>
+      </c>
+      <c r="H106" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107">
+        <v>14</v>
+      </c>
+      <c r="B107" t="s">
+        <v>165</v>
+      </c>
+      <c r="C107" s="1">
+        <v>46178</v>
+      </c>
+      <c r="D107" t="s">
+        <v>179</v>
+      </c>
+      <c r="E107" t="s">
+        <v>176</v>
+      </c>
+      <c r="F107">
+        <v>19</v>
+      </c>
+      <c r="H107" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108">
+        <v>15</v>
+      </c>
+      <c r="B108" t="s">
+        <v>164</v>
+      </c>
+      <c r="C108" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D108" t="s">
+        <v>180</v>
+      </c>
+      <c r="E108" t="s">
+        <v>187</v>
+      </c>
+      <c r="H108" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>15</v>
+      </c>
+      <c r="B109" t="s">
+        <v>164</v>
+      </c>
+      <c r="C109" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D109" t="s">
+        <v>180</v>
+      </c>
+      <c r="E109" t="s">
+        <v>188</v>
+      </c>
+      <c r="H109" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110">
+        <v>15</v>
+      </c>
+      <c r="B110" t="s">
+        <v>164</v>
+      </c>
+      <c r="C110" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D110" t="s">
+        <v>181</v>
+      </c>
+      <c r="E110" t="s">
+        <v>189</v>
+      </c>
+      <c r="H110" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111">
+        <v>15</v>
+      </c>
+      <c r="B111" t="s">
+        <v>164</v>
+      </c>
+      <c r="C111" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D111" t="s">
+        <v>181</v>
+      </c>
+      <c r="E111" t="s">
+        <v>190</v>
+      </c>
+      <c r="H111" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112">
+        <v>15</v>
+      </c>
+      <c r="B112" t="s">
+        <v>164</v>
+      </c>
+      <c r="C112" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D112" t="s">
+        <v>182</v>
+      </c>
+      <c r="E112" t="s">
+        <v>191</v>
+      </c>
+      <c r="H112" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A113">
+        <v>15</v>
+      </c>
+      <c r="B113" t="s">
+        <v>164</v>
+      </c>
+      <c r="C113" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D113" t="s">
+        <v>182</v>
+      </c>
+      <c r="E113" t="s">
+        <v>192</v>
+      </c>
+      <c r="H113" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114">
+        <v>15</v>
+      </c>
+      <c r="B114" t="s">
+        <v>164</v>
+      </c>
+      <c r="C114" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D114" t="s">
+        <v>183</v>
+      </c>
+      <c r="E114" t="s">
+        <v>193</v>
+      </c>
+      <c r="H114" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115">
+        <v>15</v>
+      </c>
+      <c r="B115" t="s">
+        <v>164</v>
+      </c>
+      <c r="C115" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D115" t="s">
+        <v>183</v>
+      </c>
+      <c r="E115" t="s">
+        <v>194</v>
+      </c>
+      <c r="H115" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116">
+        <v>15</v>
+      </c>
+      <c r="B116" t="s">
+        <v>164</v>
+      </c>
+      <c r="C116" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D116" t="s">
+        <v>184</v>
+      </c>
+      <c r="E116" t="s">
+        <v>195</v>
+      </c>
+      <c r="H116" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117">
+        <v>15</v>
+      </c>
+      <c r="B117" t="s">
+        <v>164</v>
+      </c>
+      <c r="C117" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D117" t="s">
+        <v>184</v>
+      </c>
+      <c r="E117" t="s">
+        <v>196</v>
+      </c>
+      <c r="H117" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>15</v>
+      </c>
+      <c r="B118" t="s">
+        <v>164</v>
+      </c>
+      <c r="C118" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D118" t="s">
+        <v>185</v>
+      </c>
+      <c r="E118" t="s">
+        <v>197</v>
+      </c>
+      <c r="H118" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119">
+        <v>15</v>
+      </c>
+      <c r="B119" t="s">
+        <v>164</v>
+      </c>
+      <c r="C119" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D119" t="s">
+        <v>185</v>
+      </c>
+      <c r="E119" t="s">
+        <v>198</v>
+      </c>
+      <c r="H119" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120">
+        <v>15</v>
+      </c>
+      <c r="B120" t="s">
+        <v>164</v>
+      </c>
+      <c r="C120" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D120" t="s">
+        <v>186</v>
+      </c>
+      <c r="E120" t="s">
+        <v>199</v>
+      </c>
+      <c r="H120" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121">
+        <v>15</v>
+      </c>
+      <c r="B121" t="s">
+        <v>164</v>
+      </c>
+      <c r="C121" s="1">
+        <v>46185</v>
+      </c>
+      <c r="D121" t="s">
+        <v>186</v>
+      </c>
+      <c r="E121" t="s">
+        <v>200</v>
+      </c>
+      <c r="H121" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dessert matchup pt 2
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D82D16-9EF8-483E-905F-37852E37AD92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220CDE41-E70A-427F-9DD5-87D4493CD462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="-96" windowWidth="23232" windowHeight="13872" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="234">
   <si>
     <t>option</t>
   </si>
@@ -44,9 +44,6 @@
     <t>series</t>
   </si>
   <si>
-    <t>week</t>
-  </si>
-  <si>
     <t>question</t>
   </si>
   <si>
@@ -639,6 +636,108 @@
   </si>
   <si>
     <t>"Bless your heart"</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Dessert Match-Ups Part II</t>
+  </si>
+  <si>
+    <t>Cookie</t>
+  </si>
+  <si>
+    <t>Macaron</t>
+  </si>
+  <si>
+    <t>Macaroon</t>
+  </si>
+  <si>
+    <t>Tart/Torte</t>
+  </si>
+  <si>
+    <t>Fruit Tart</t>
+  </si>
+  <si>
+    <t>Chocolate Torte</t>
+  </si>
+  <si>
+    <t>Cinnamon</t>
+  </si>
+  <si>
+    <t>Churro</t>
+  </si>
+  <si>
+    <t>Cinnamon Bun</t>
+  </si>
+  <si>
+    <t>Flan</t>
+  </si>
+  <si>
+    <t>Panna Cotta</t>
+  </si>
+  <si>
+    <t>Chilled and Molded</t>
+  </si>
+  <si>
+    <t>Summer Treat</t>
+  </si>
+  <si>
+    <t>Ice Cream Sandwich</t>
+  </si>
+  <si>
+    <t>Popsicle</t>
+  </si>
+  <si>
+    <t>Sun Protection</t>
+  </si>
+  <si>
+    <t>Sunscreen</t>
+  </si>
+  <si>
+    <t>Shades</t>
+  </si>
+  <si>
+    <t>Hat</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Burn Care</t>
+  </si>
+  <si>
+    <t>Lotion</t>
+  </si>
+  <si>
+    <t>Spray</t>
+  </si>
+  <si>
+    <t>Aviator</t>
+  </si>
+  <si>
+    <t>Wayfarer</t>
+  </si>
+  <si>
+    <t>Baseball Cap</t>
+  </si>
+  <si>
+    <t>Bucket Hat</t>
+  </si>
+  <si>
+    <t>Wide-brimmed Floppy Hat</t>
+  </si>
+  <si>
+    <t>Long Sleeves</t>
+  </si>
+  <si>
+    <t>Reapply Sunscreen</t>
+  </si>
+  <si>
+    <t>Aloe</t>
+  </si>
+  <si>
+    <t>Moisturizing Lotion</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -1025,28 +1124,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="G1" t="s">
-        <v>91</v>
-      </c>
       <c r="H1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1054,22 +1153,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C2" s="1">
         <v>45992</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2">
         <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1077,22 +1176,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C3" s="1">
         <v>45992</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3">
         <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1100,22 +1199,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C4" s="1">
         <v>45999</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
         <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1123,22 +1222,22 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C5" s="1">
         <v>45999</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5">
         <v>28</v>
       </c>
       <c r="H5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1146,22 +1245,22 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C6" s="1">
         <v>46006</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6">
         <v>6</v>
       </c>
       <c r="H6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1169,22 +1268,22 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C7" s="1">
         <v>46006</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7">
         <v>10</v>
       </c>
       <c r="H7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1192,22 +1291,22 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C8" s="1">
         <v>46006</v>
       </c>
       <c r="D8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F8">
         <v>3</v>
       </c>
       <c r="H8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1215,22 +1314,22 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C9" s="1">
         <v>46006</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F9">
         <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1238,22 +1337,22 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C10" s="1">
         <v>46013</v>
       </c>
       <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
         <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
       </c>
       <c r="F10">
         <v>21</v>
       </c>
       <c r="H10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1261,22 +1360,22 @@
         <v>4</v>
       </c>
       <c r="B11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C11" s="1">
         <v>46013</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F11">
         <v>4</v>
       </c>
       <c r="H11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1284,22 +1383,22 @@
         <v>5</v>
       </c>
       <c r="B12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C12" s="1">
         <v>46027</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F12">
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1307,22 +1406,22 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C13" s="1">
         <v>46027</v>
       </c>
       <c r="D13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13">
         <v>17</v>
       </c>
       <c r="H13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1330,22 +1429,22 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="1">
         <v>46034</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F14">
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1353,22 +1452,22 @@
         <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C15" s="1">
         <v>46034</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F15">
         <v>13</v>
       </c>
       <c r="H15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1376,22 +1475,22 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C16" s="1">
         <v>46042</v>
       </c>
       <c r="D16" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F16">
         <v>24</v>
       </c>
       <c r="H16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1399,22 +1498,22 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C17" s="1">
         <v>46042</v>
       </c>
       <c r="D17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17">
         <v>9</v>
       </c>
       <c r="H17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1422,22 +1521,22 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C18" s="1">
         <v>46042</v>
       </c>
       <c r="D18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F18">
         <v>24</v>
       </c>
       <c r="H18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1445,22 +1544,22 @@
         <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C19" s="1">
         <v>46042</v>
       </c>
       <c r="D19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F19">
         <v>9</v>
       </c>
       <c r="H19" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1468,22 +1567,22 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C20" s="1">
         <v>46042</v>
       </c>
       <c r="D20" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F20">
         <v>10</v>
       </c>
       <c r="H20" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1491,22 +1590,22 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C21" s="1">
         <v>46042</v>
       </c>
       <c r="D21" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F21">
         <v>23</v>
       </c>
       <c r="H21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1514,22 +1613,22 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C22" s="1">
         <v>46042</v>
       </c>
       <c r="D22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F22">
         <v>24</v>
       </c>
       <c r="H22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1537,22 +1636,22 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C23" s="1">
         <v>46042</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F23">
         <v>9</v>
       </c>
       <c r="H23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1560,22 +1659,22 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C24" s="1">
         <v>46063</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F24">
         <v>19</v>
       </c>
       <c r="H24" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1583,22 +1682,22 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C25" s="1">
         <v>46063</v>
       </c>
       <c r="D25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F25">
         <v>18</v>
       </c>
       <c r="H25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1606,22 +1705,22 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C26" s="1">
         <v>46063</v>
       </c>
       <c r="D26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F26">
         <v>25</v>
       </c>
       <c r="H26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1629,22 +1728,22 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C27" s="1">
         <v>46063</v>
       </c>
       <c r="D27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F27">
         <v>7</v>
       </c>
       <c r="H27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1652,22 +1751,22 @@
         <v>7</v>
       </c>
       <c r="B28" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C28" s="1">
         <v>46063</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F28">
         <v>18</v>
       </c>
       <c r="H28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1675,22 +1774,22 @@
         <v>7</v>
       </c>
       <c r="B29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C29" s="1">
         <v>46063</v>
       </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F29">
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1698,22 +1797,22 @@
         <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C30" s="1">
         <v>46063</v>
       </c>
       <c r="D30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F30">
         <v>8</v>
       </c>
       <c r="H30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1721,22 +1820,22 @@
         <v>7</v>
       </c>
       <c r="B31" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C31" s="1">
         <v>46063</v>
       </c>
       <c r="D31" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F31">
         <v>20</v>
       </c>
       <c r="H31" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1744,22 +1843,22 @@
         <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C32" s="1">
         <v>46076</v>
       </c>
       <c r="D32" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F32">
         <v>11</v>
       </c>
       <c r="H32" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1767,22 +1866,22 @@
         <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C33" s="1">
         <v>46076</v>
       </c>
       <c r="D33" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F33">
         <v>20</v>
       </c>
       <c r="H33" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1790,22 +1889,22 @@
         <v>8</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C34" s="1">
         <v>46076</v>
       </c>
       <c r="D34" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E34" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F34">
         <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1813,22 +1912,22 @@
         <v>8</v>
       </c>
       <c r="B35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C35" s="1">
         <v>46076</v>
       </c>
       <c r="D35" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E35" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F35">
         <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -1836,22 +1935,22 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C36" s="1">
         <v>46076</v>
       </c>
       <c r="D36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F36">
         <v>17</v>
       </c>
       <c r="H36" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -1859,22 +1958,22 @@
         <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C37" s="1">
         <v>46076</v>
       </c>
       <c r="D37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E37" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F37">
         <v>7</v>
       </c>
       <c r="H37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -1882,22 +1981,22 @@
         <v>8</v>
       </c>
       <c r="B38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C38" s="1">
         <v>46076</v>
       </c>
       <c r="D38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F38">
         <v>6</v>
       </c>
       <c r="H38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -1905,22 +2004,22 @@
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C39" s="1">
         <v>46076</v>
       </c>
       <c r="D39" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F39">
         <v>18</v>
       </c>
       <c r="H39" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1928,22 +2027,22 @@
         <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C40" s="1">
         <v>46076</v>
       </c>
       <c r="D40" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E40" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F40">
         <v>18</v>
       </c>
       <c r="H40" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -1951,22 +2050,22 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C41" s="1">
         <v>46076</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F41">
         <v>4</v>
       </c>
       <c r="H41" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1974,22 +2073,22 @@
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C42" s="1">
         <v>46087</v>
       </c>
       <c r="D42" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E42" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F42">
         <v>23</v>
       </c>
       <c r="H42" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1997,22 +2096,22 @@
         <v>9</v>
       </c>
       <c r="B43" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C43" s="1">
         <v>46087</v>
       </c>
       <c r="D43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F43">
         <v>15</v>
       </c>
       <c r="H43" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2020,22 +2119,22 @@
         <v>9</v>
       </c>
       <c r="B44" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C44" s="1">
         <v>46087</v>
       </c>
       <c r="D44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F44">
         <v>21</v>
       </c>
       <c r="H44" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2043,22 +2142,22 @@
         <v>9</v>
       </c>
       <c r="B45" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C45" s="1">
         <v>46087</v>
       </c>
       <c r="D45" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F45">
         <v>20</v>
       </c>
       <c r="H45" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2066,22 +2165,22 @@
         <v>9</v>
       </c>
       <c r="B46" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C46" s="1">
         <v>46087</v>
       </c>
       <c r="D46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F46">
         <v>10</v>
       </c>
       <c r="H46" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2089,22 +2188,22 @@
         <v>9</v>
       </c>
       <c r="B47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C47" s="1">
         <v>46087</v>
       </c>
       <c r="D47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F47">
         <v>20</v>
       </c>
       <c r="H47" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2112,22 +2211,22 @@
         <v>9</v>
       </c>
       <c r="B48" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C48" s="1">
         <v>46087</v>
       </c>
       <c r="D48" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F48">
         <v>6</v>
       </c>
       <c r="H48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2135,22 +2234,22 @@
         <v>9</v>
       </c>
       <c r="B49" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C49" s="1">
         <v>46087</v>
       </c>
       <c r="D49" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E49" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F49">
         <v>14</v>
       </c>
       <c r="H49" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2158,22 +2257,22 @@
         <v>9</v>
       </c>
       <c r="B50" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C50" s="1">
         <v>46087</v>
       </c>
       <c r="D50" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E50" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F50">
         <v>6</v>
       </c>
       <c r="H50" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2181,22 +2280,22 @@
         <v>9</v>
       </c>
       <c r="B51" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C51" s="1">
         <v>46087</v>
       </c>
       <c r="D51" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F51">
         <v>34</v>
       </c>
       <c r="H51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2204,22 +2303,22 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C52" s="1">
         <v>46099</v>
       </c>
       <c r="D52" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F52">
         <v>25</v>
       </c>
       <c r="H52" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2227,22 +2326,22 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C53" s="1">
         <v>46099</v>
       </c>
       <c r="D53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F53">
         <v>13</v>
       </c>
       <c r="H53" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2250,22 +2349,22 @@
         <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C54" s="1">
         <v>46099</v>
       </c>
       <c r="D54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F54">
         <v>8</v>
       </c>
       <c r="H54" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2273,22 +2372,22 @@
         <v>10</v>
       </c>
       <c r="B55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C55" s="1">
         <v>46099</v>
       </c>
       <c r="D55" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F55">
         <v>29</v>
       </c>
       <c r="H55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2296,22 +2395,22 @@
         <v>10</v>
       </c>
       <c r="B56" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C56" s="1">
         <v>46099</v>
       </c>
       <c r="D56" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F56">
         <v>21</v>
       </c>
       <c r="H56" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2319,22 +2418,22 @@
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C57" s="1">
         <v>46099</v>
       </c>
       <c r="D57" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F57">
         <v>14</v>
       </c>
       <c r="H57" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2342,22 +2441,22 @@
         <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C58" s="1">
         <v>46099</v>
       </c>
       <c r="D58" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E58" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F58">
         <v>22</v>
       </c>
       <c r="H58" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -2365,22 +2464,22 @@
         <v>10</v>
       </c>
       <c r="B59" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C59" s="1">
         <v>46099</v>
       </c>
       <c r="D59" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E59" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F59">
         <v>8</v>
       </c>
       <c r="H59" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -2388,22 +2487,22 @@
         <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C60" s="1">
         <v>46099</v>
       </c>
       <c r="D60" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E60" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F60">
         <v>7</v>
       </c>
       <c r="H60" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -2411,22 +2510,22 @@
         <v>10</v>
       </c>
       <c r="B61" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C61" s="1">
         <v>46099</v>
       </c>
       <c r="D61" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F61">
         <v>28</v>
       </c>
       <c r="H61" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -2434,22 +2533,22 @@
         <v>11</v>
       </c>
       <c r="B62" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C62" s="1">
         <v>46125</v>
       </c>
       <c r="D62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E62" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F62">
         <v>27</v>
       </c>
       <c r="H62" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -2457,22 +2556,22 @@
         <v>11</v>
       </c>
       <c r="B63" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C63" s="1">
         <v>46125</v>
       </c>
       <c r="D63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E63" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F63">
         <v>22</v>
       </c>
       <c r="H63" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -2480,22 +2579,22 @@
         <v>11</v>
       </c>
       <c r="B64" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C64" s="1">
         <v>46125</v>
       </c>
       <c r="D64" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E64" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F64">
         <v>26</v>
       </c>
       <c r="H64" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
@@ -2503,22 +2602,22 @@
         <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C65" s="1">
         <v>46125</v>
       </c>
       <c r="D65" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F65">
         <v>19</v>
       </c>
       <c r="H65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
@@ -2526,22 +2625,22 @@
         <v>11</v>
       </c>
       <c r="B66" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C66" s="1">
         <v>46125</v>
       </c>
       <c r="D66" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E66" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F66">
         <v>35</v>
       </c>
       <c r="H66" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
@@ -2549,22 +2648,22 @@
         <v>11</v>
       </c>
       <c r="B67" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C67" s="1">
         <v>46125</v>
       </c>
       <c r="D67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E67" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F67">
         <v>10</v>
       </c>
       <c r="H67" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
@@ -2572,22 +2671,22 @@
         <v>11</v>
       </c>
       <c r="B68" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C68" s="1">
         <v>46125</v>
       </c>
       <c r="D68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E68" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F68">
         <v>20</v>
       </c>
       <c r="H68" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
@@ -2595,22 +2694,22 @@
         <v>11</v>
       </c>
       <c r="B69" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C69" s="1">
         <v>46125</v>
       </c>
       <c r="D69" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E69" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F69">
         <v>28</v>
       </c>
       <c r="H69" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2618,22 +2717,22 @@
         <v>11</v>
       </c>
       <c r="B70" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C70" s="1">
         <v>46125</v>
       </c>
       <c r="D70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E70" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F70">
         <v>28</v>
       </c>
       <c r="H70" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2641,22 +2740,22 @@
         <v>11</v>
       </c>
       <c r="B71" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C71" s="1">
         <v>46125</v>
       </c>
       <c r="D71" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E71" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F71">
         <v>21</v>
       </c>
       <c r="H71" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2664,22 +2763,22 @@
         <v>11</v>
       </c>
       <c r="B72" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C72" s="1">
         <v>46125</v>
       </c>
       <c r="D72" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E72" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F72">
         <v>32</v>
       </c>
       <c r="H72" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2687,22 +2786,22 @@
         <v>11</v>
       </c>
       <c r="B73" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C73" s="1">
         <v>46125</v>
       </c>
       <c r="D73" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E73" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F73">
         <v>11</v>
       </c>
       <c r="H73" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2710,22 +2809,22 @@
         <v>11</v>
       </c>
       <c r="B74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C74" s="1">
         <v>46125</v>
       </c>
       <c r="D74" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E74" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F74">
         <v>34</v>
       </c>
       <c r="H74" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2733,22 +2832,22 @@
         <v>11</v>
       </c>
       <c r="B75" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C75" s="1">
         <v>46125</v>
       </c>
       <c r="D75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F75">
         <v>9</v>
       </c>
       <c r="H75" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2756,16 +2855,16 @@
         <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C76" s="1">
         <v>46150</v>
       </c>
       <c r="D76" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E76" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F76">
         <v>7</v>
@@ -2774,7 +2873,7 @@
         <v>6</v>
       </c>
       <c r="H76" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -2782,16 +2881,16 @@
         <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C77" s="1">
         <v>46150</v>
       </c>
       <c r="D77" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E77" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F77">
         <v>32</v>
@@ -2800,7 +2899,7 @@
         <v>27</v>
       </c>
       <c r="H77" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -2808,16 +2907,16 @@
         <v>12</v>
       </c>
       <c r="B78" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C78" s="1">
         <v>46150</v>
       </c>
       <c r="D78" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E78" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F78">
         <v>19</v>
@@ -2826,7 +2925,7 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2834,16 +2933,16 @@
         <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C79" s="1">
         <v>46150</v>
       </c>
       <c r="D79" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E79" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F79">
         <v>25</v>
@@ -2852,7 +2951,7 @@
         <v>21</v>
       </c>
       <c r="H79" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -2860,16 +2959,16 @@
         <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C80" s="1">
         <v>46150</v>
       </c>
       <c r="D80" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E80" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F80">
         <v>11</v>
@@ -2878,7 +2977,7 @@
         <v>12</v>
       </c>
       <c r="H80" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
@@ -2886,16 +2985,16 @@
         <v>12</v>
       </c>
       <c r="B81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C81" s="1">
         <v>46150</v>
       </c>
       <c r="D81" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E81" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F81">
         <v>27</v>
@@ -2904,7 +3003,7 @@
         <v>23</v>
       </c>
       <c r="H81" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -2912,16 +3011,16 @@
         <v>12</v>
       </c>
       <c r="B82" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C82" s="1">
         <v>46150</v>
       </c>
       <c r="D82" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E82" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F82">
         <v>17</v>
@@ -2930,7 +3029,7 @@
         <v>20</v>
       </c>
       <c r="H82" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -2938,16 +3037,16 @@
         <v>12</v>
       </c>
       <c r="B83" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C83" s="1">
         <v>46150</v>
       </c>
       <c r="D83" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E83" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F83">
         <v>21</v>
@@ -2956,7 +3055,7 @@
         <v>14</v>
       </c>
       <c r="H83" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -2964,16 +3063,16 @@
         <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C84" s="1">
         <v>46164</v>
       </c>
       <c r="D84" t="s">
+        <v>125</v>
+      </c>
+      <c r="E84" t="s">
         <v>126</v>
-      </c>
-      <c r="E84" t="s">
-        <v>127</v>
       </c>
       <c r="F84">
         <v>24</v>
@@ -2982,7 +3081,7 @@
         <v>21</v>
       </c>
       <c r="H84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -2990,16 +3089,16 @@
         <v>13</v>
       </c>
       <c r="B85" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C85" s="1">
         <v>46164</v>
       </c>
       <c r="D85" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E85" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F85">
         <v>10</v>
@@ -3008,7 +3107,7 @@
         <v>8</v>
       </c>
       <c r="H85" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3016,16 +3115,16 @@
         <v>13</v>
       </c>
       <c r="B86" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C86" s="1">
         <v>46164</v>
       </c>
       <c r="D86" t="s">
+        <v>128</v>
+      </c>
+      <c r="E86" t="s">
         <v>129</v>
-      </c>
-      <c r="E86" t="s">
-        <v>130</v>
       </c>
       <c r="F86">
         <v>18</v>
@@ -3034,7 +3133,7 @@
         <v>16</v>
       </c>
       <c r="H86" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3042,16 +3141,16 @@
         <v>13</v>
       </c>
       <c r="B87" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C87" s="1">
         <v>46164</v>
       </c>
       <c r="D87" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E87" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F87">
         <v>16</v>
@@ -3060,7 +3159,7 @@
         <v>11</v>
       </c>
       <c r="H87" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3068,16 +3167,16 @@
         <v>13</v>
       </c>
       <c r="B88" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C88" s="1">
         <v>46164</v>
       </c>
       <c r="D88" t="s">
+        <v>131</v>
+      </c>
+      <c r="E88" t="s">
         <v>132</v>
-      </c>
-      <c r="E88" t="s">
-        <v>133</v>
       </c>
       <c r="F88">
         <v>21</v>
@@ -3086,7 +3185,7 @@
         <v>14</v>
       </c>
       <c r="H88" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3094,16 +3193,16 @@
         <v>13</v>
       </c>
       <c r="B89" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C89" s="1">
         <v>46164</v>
       </c>
       <c r="D89" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E89" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F89">
         <v>12</v>
@@ -3112,7 +3211,7 @@
         <v>14</v>
       </c>
       <c r="H89" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -3120,16 +3219,16 @@
         <v>13</v>
       </c>
       <c r="B90" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C90" s="1">
         <v>46164</v>
       </c>
       <c r="D90" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E90" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F90">
         <v>17</v>
@@ -3138,7 +3237,7 @@
         <v>16</v>
       </c>
       <c r="H90" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -3146,16 +3245,16 @@
         <v>13</v>
       </c>
       <c r="B91" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C91" s="1">
         <v>46164</v>
       </c>
       <c r="D91" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E91" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F91">
         <v>16</v>
@@ -3164,7 +3263,7 @@
         <v>12</v>
       </c>
       <c r="H91" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -3172,16 +3271,16 @@
         <v>13</v>
       </c>
       <c r="B92" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C92" s="1">
         <v>46164</v>
       </c>
       <c r="D92" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E92" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F92">
         <v>22</v>
@@ -3190,7 +3289,7 @@
         <v>19</v>
       </c>
       <c r="H92" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -3198,16 +3297,16 @@
         <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C93" s="1">
         <v>46164</v>
       </c>
       <c r="D93" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F93">
         <v>12</v>
@@ -3216,7 +3315,7 @@
         <v>9</v>
       </c>
       <c r="H93" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -3224,16 +3323,16 @@
         <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C94" s="1">
         <v>46164</v>
       </c>
       <c r="D94" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E94" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F94">
         <v>9</v>
@@ -3242,7 +3341,7 @@
         <v>11</v>
       </c>
       <c r="H94" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -3250,16 +3349,16 @@
         <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C95" s="1">
         <v>46164</v>
       </c>
       <c r="D95" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E95" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F95">
         <v>25</v>
@@ -3268,7 +3367,7 @@
         <v>19</v>
       </c>
       <c r="H95" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.25">
@@ -3276,16 +3375,16 @@
         <v>13</v>
       </c>
       <c r="B96" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C96" s="1">
         <v>46164</v>
       </c>
       <c r="D96" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E96" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F96">
         <v>24</v>
@@ -3294,7 +3393,7 @@
         <v>18</v>
       </c>
       <c r="H96" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3302,16 +3401,16 @@
         <v>13</v>
       </c>
       <c r="B97" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C97" s="1">
         <v>46164</v>
       </c>
       <c r="D97" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E97" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F97">
         <v>10</v>
@@ -3320,7 +3419,7 @@
         <v>11</v>
       </c>
       <c r="H97" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
@@ -3328,22 +3427,25 @@
         <v>14</v>
       </c>
       <c r="B98" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C98" s="1">
         <v>46178</v>
       </c>
       <c r="D98" t="s">
+        <v>165</v>
+      </c>
+      <c r="E98" t="s">
         <v>166</v>
-      </c>
-      <c r="E98" t="s">
-        <v>167</v>
       </c>
       <c r="F98">
         <v>19</v>
       </c>
+      <c r="G98">
+        <v>13</v>
+      </c>
       <c r="H98" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.25">
@@ -3351,22 +3453,25 @@
         <v>14</v>
       </c>
       <c r="B99" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C99" s="1">
         <v>46178</v>
       </c>
       <c r="D99" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E99" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F99">
         <v>32</v>
       </c>
+      <c r="G99">
+        <v>10</v>
+      </c>
       <c r="H99" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.25">
@@ -3374,22 +3479,25 @@
         <v>14</v>
       </c>
       <c r="B100" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C100" s="1">
         <v>46178</v>
       </c>
       <c r="D100" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E100" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F100">
         <v>28</v>
       </c>
+      <c r="G100">
+        <v>16</v>
+      </c>
       <c r="H100" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.25">
@@ -3397,22 +3505,25 @@
         <v>14</v>
       </c>
       <c r="B101" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C101" s="1">
         <v>46178</v>
       </c>
       <c r="D101" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E101" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F101">
         <v>22</v>
       </c>
+      <c r="G101">
+        <v>5</v>
+      </c>
       <c r="H101" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.25">
@@ -3420,22 +3531,25 @@
         <v>14</v>
       </c>
       <c r="B102" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C102" s="1">
         <v>46178</v>
       </c>
       <c r="D102" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E102" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F102">
         <v>25</v>
       </c>
+      <c r="G102">
+        <v>10</v>
+      </c>
       <c r="H102" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.25">
@@ -3443,22 +3557,25 @@
         <v>14</v>
       </c>
       <c r="B103" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C103" s="1">
         <v>46178</v>
       </c>
       <c r="D103" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E103" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F103">
         <v>27</v>
       </c>
+      <c r="G103">
+        <v>11</v>
+      </c>
       <c r="H103" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -3466,22 +3583,25 @@
         <v>14</v>
       </c>
       <c r="B104" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C104" s="1">
         <v>46178</v>
       </c>
       <c r="D104" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E104" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F104">
         <v>44</v>
       </c>
+      <c r="G104">
+        <v>21</v>
+      </c>
       <c r="H104" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
@@ -3489,22 +3609,25 @@
         <v>14</v>
       </c>
       <c r="B105" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C105" s="1">
         <v>46178</v>
       </c>
       <c r="D105" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E105" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F105">
         <v>9</v>
       </c>
+      <c r="G105">
+        <v>2</v>
+      </c>
       <c r="H105" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
@@ -3512,22 +3635,25 @@
         <v>14</v>
       </c>
       <c r="B106" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C106" s="1">
         <v>46178</v>
       </c>
       <c r="D106" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E106" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F106">
         <v>30</v>
       </c>
+      <c r="G106">
+        <v>15</v>
+      </c>
       <c r="H106" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
@@ -3535,22 +3661,25 @@
         <v>14</v>
       </c>
       <c r="B107" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C107" s="1">
         <v>46178</v>
       </c>
       <c r="D107" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E107" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F107">
         <v>19</v>
       </c>
+      <c r="G107">
+        <v>7</v>
+      </c>
       <c r="H107" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
@@ -3558,19 +3687,25 @@
         <v>15</v>
       </c>
       <c r="B108" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C108" s="1">
         <v>46185</v>
       </c>
       <c r="D108" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E108" t="s">
-        <v>187</v>
+        <v>186</v>
+      </c>
+      <c r="F108">
+        <v>23</v>
+      </c>
+      <c r="G108">
+        <v>13</v>
       </c>
       <c r="H108" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
@@ -3578,19 +3713,25 @@
         <v>15</v>
       </c>
       <c r="B109" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C109" s="1">
         <v>46185</v>
       </c>
       <c r="D109" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E109" t="s">
-        <v>188</v>
+        <v>187</v>
+      </c>
+      <c r="F109">
+        <v>8</v>
+      </c>
+      <c r="G109">
+        <v>9</v>
       </c>
       <c r="H109" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
@@ -3598,19 +3739,25 @@
         <v>15</v>
       </c>
       <c r="B110" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C110" s="1">
         <v>46185</v>
       </c>
       <c r="D110" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E110" t="s">
-        <v>189</v>
+        <v>188</v>
+      </c>
+      <c r="F110">
+        <v>14</v>
+      </c>
+      <c r="G110">
+        <v>14</v>
       </c>
       <c r="H110" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.25">
@@ -3618,19 +3765,25 @@
         <v>15</v>
       </c>
       <c r="B111" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C111" s="1">
         <v>46185</v>
       </c>
       <c r="D111" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E111" t="s">
-        <v>190</v>
+        <v>189</v>
+      </c>
+      <c r="F111">
+        <v>18</v>
+      </c>
+      <c r="G111">
+        <v>9</v>
       </c>
       <c r="H111" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -3638,19 +3791,25 @@
         <v>15</v>
       </c>
       <c r="B112" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C112" s="1">
         <v>46185</v>
       </c>
       <c r="D112" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E112" t="s">
-        <v>191</v>
+        <v>190</v>
+      </c>
+      <c r="F112">
+        <v>4</v>
+      </c>
+      <c r="G112">
+        <v>6</v>
       </c>
       <c r="H112" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
@@ -3658,19 +3817,25 @@
         <v>15</v>
       </c>
       <c r="B113" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C113" s="1">
         <v>46185</v>
       </c>
       <c r="D113" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E113" t="s">
-        <v>192</v>
+        <v>191</v>
+      </c>
+      <c r="F113">
+        <v>22</v>
+      </c>
+      <c r="G113">
+        <v>15</v>
       </c>
       <c r="H113" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
@@ -3678,19 +3843,25 @@
         <v>15</v>
       </c>
       <c r="B114" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C114" s="1">
         <v>46185</v>
       </c>
       <c r="D114" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E114" t="s">
-        <v>193</v>
+        <v>192</v>
+      </c>
+      <c r="F114">
+        <v>25</v>
+      </c>
+      <c r="G114">
+        <v>16</v>
       </c>
       <c r="H114" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
@@ -3698,19 +3869,25 @@
         <v>15</v>
       </c>
       <c r="B115" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C115" s="1">
         <v>46185</v>
       </c>
       <c r="D115" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E115" t="s">
-        <v>194</v>
+        <v>193</v>
+      </c>
+      <c r="F115">
+        <v>5</v>
+      </c>
+      <c r="G115">
+        <v>7</v>
       </c>
       <c r="H115" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
@@ -3718,19 +3895,25 @@
         <v>15</v>
       </c>
       <c r="B116" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C116" s="1">
         <v>46185</v>
       </c>
       <c r="D116" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E116" t="s">
-        <v>195</v>
+        <v>194</v>
+      </c>
+      <c r="F116">
+        <v>22</v>
+      </c>
+      <c r="G116">
+        <v>16</v>
       </c>
       <c r="H116" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
@@ -3738,19 +3921,25 @@
         <v>15</v>
       </c>
       <c r="B117" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C117" s="1">
         <v>46185</v>
       </c>
       <c r="D117" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E117" t="s">
-        <v>196</v>
+        <v>195</v>
+      </c>
+      <c r="F117">
+        <v>10</v>
+      </c>
+      <c r="G117">
+        <v>7</v>
       </c>
       <c r="H117" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
@@ -3758,19 +3947,25 @@
         <v>15</v>
       </c>
       <c r="B118" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C118" s="1">
         <v>46185</v>
       </c>
       <c r="D118" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E118" t="s">
-        <v>197</v>
+        <v>196</v>
+      </c>
+      <c r="F118">
+        <v>17</v>
+      </c>
+      <c r="G118">
+        <v>13</v>
       </c>
       <c r="H118" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
@@ -3778,19 +3973,25 @@
         <v>15</v>
       </c>
       <c r="B119" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C119" s="1">
         <v>46185</v>
       </c>
       <c r="D119" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E119" t="s">
-        <v>198</v>
+        <v>197</v>
+      </c>
+      <c r="F119">
+        <v>10</v>
+      </c>
+      <c r="G119">
+        <v>8</v>
       </c>
       <c r="H119" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -3798,19 +3999,25 @@
         <v>15</v>
       </c>
       <c r="B120" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C120" s="1">
         <v>46185</v>
       </c>
       <c r="D120" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E120" t="s">
-        <v>199</v>
+        <v>198</v>
+      </c>
+      <c r="F120">
+        <v>15</v>
+      </c>
+      <c r="G120">
+        <v>15</v>
       </c>
       <c r="H120" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -3818,19 +4025,505 @@
         <v>15</v>
       </c>
       <c r="B121" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C121" s="1">
         <v>46185</v>
       </c>
       <c r="D121" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E121" t="s">
-        <v>200</v>
+        <v>199</v>
+      </c>
+      <c r="F121">
+        <v>16</v>
+      </c>
+      <c r="G121">
+        <v>12</v>
       </c>
       <c r="H121" t="s">
-        <v>150</v>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122">
+        <v>16</v>
+      </c>
+      <c r="B122" t="s">
+        <v>201</v>
+      </c>
+      <c r="C122" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D122" t="s">
+        <v>202</v>
+      </c>
+      <c r="E122" t="s">
+        <v>203</v>
+      </c>
+      <c r="F122">
+        <v>11</v>
+      </c>
+      <c r="G122">
+        <v>8</v>
+      </c>
+      <c r="H122" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123">
+        <v>16</v>
+      </c>
+      <c r="B123" t="s">
+        <v>201</v>
+      </c>
+      <c r="C123" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D123" t="s">
+        <v>202</v>
+      </c>
+      <c r="E123" t="s">
+        <v>204</v>
+      </c>
+      <c r="F123">
+        <v>17</v>
+      </c>
+      <c r="G123">
+        <v>6</v>
+      </c>
+      <c r="H123" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A124">
+        <v>16</v>
+      </c>
+      <c r="B124" t="s">
+        <v>201</v>
+      </c>
+      <c r="C124" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D124" t="s">
+        <v>205</v>
+      </c>
+      <c r="E124" t="s">
+        <v>206</v>
+      </c>
+      <c r="F124">
+        <v>19</v>
+      </c>
+      <c r="G124">
+        <v>7</v>
+      </c>
+      <c r="H124" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125">
+        <v>16</v>
+      </c>
+      <c r="B125" t="s">
+        <v>201</v>
+      </c>
+      <c r="C125" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D125" t="s">
+        <v>205</v>
+      </c>
+      <c r="E125" t="s">
+        <v>207</v>
+      </c>
+      <c r="F125">
+        <v>13</v>
+      </c>
+      <c r="G125">
+        <v>8</v>
+      </c>
+      <c r="H125" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>16</v>
+      </c>
+      <c r="B126" t="s">
+        <v>201</v>
+      </c>
+      <c r="C126" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D126" t="s">
+        <v>208</v>
+      </c>
+      <c r="E126" t="s">
+        <v>209</v>
+      </c>
+      <c r="F126">
+        <v>16</v>
+      </c>
+      <c r="G126">
+        <v>7</v>
+      </c>
+      <c r="H126" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127">
+        <v>16</v>
+      </c>
+      <c r="B127" t="s">
+        <v>201</v>
+      </c>
+      <c r="C127" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D127" t="s">
+        <v>208</v>
+      </c>
+      <c r="E127" t="s">
+        <v>210</v>
+      </c>
+      <c r="F127">
+        <v>15</v>
+      </c>
+      <c r="G127">
+        <v>8</v>
+      </c>
+      <c r="H127" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128">
+        <v>16</v>
+      </c>
+      <c r="B128" t="s">
+        <v>201</v>
+      </c>
+      <c r="C128" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D128" t="s">
+        <v>213</v>
+      </c>
+      <c r="E128" t="s">
+        <v>211</v>
+      </c>
+      <c r="F128">
+        <v>22</v>
+      </c>
+      <c r="G128">
+        <v>8</v>
+      </c>
+      <c r="H128" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129">
+        <v>16</v>
+      </c>
+      <c r="B129" t="s">
+        <v>201</v>
+      </c>
+      <c r="C129" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D129" t="s">
+        <v>213</v>
+      </c>
+      <c r="E129" t="s">
+        <v>212</v>
+      </c>
+      <c r="F129">
+        <v>7</v>
+      </c>
+      <c r="G129">
+        <v>6</v>
+      </c>
+      <c r="H129" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130">
+        <v>16</v>
+      </c>
+      <c r="B130" t="s">
+        <v>201</v>
+      </c>
+      <c r="C130" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D130" t="s">
+        <v>214</v>
+      </c>
+      <c r="E130" t="s">
+        <v>215</v>
+      </c>
+      <c r="F130">
+        <v>23</v>
+      </c>
+      <c r="G130">
+        <v>13</v>
+      </c>
+      <c r="H130" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131">
+        <v>16</v>
+      </c>
+      <c r="B131" t="s">
+        <v>201</v>
+      </c>
+      <c r="C131" s="1">
+        <v>46192</v>
+      </c>
+      <c r="D131" t="s">
+        <v>214</v>
+      </c>
+      <c r="E131" t="s">
+        <v>216</v>
+      </c>
+      <c r="F131">
+        <v>8</v>
+      </c>
+      <c r="G131">
+        <v>3</v>
+      </c>
+      <c r="H131" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132">
+        <v>17</v>
+      </c>
+      <c r="B132" t="s">
+        <v>217</v>
+      </c>
+      <c r="C132" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D132" t="s">
+        <v>218</v>
+      </c>
+      <c r="E132" t="s">
+        <v>223</v>
+      </c>
+      <c r="H132" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133">
+        <v>17</v>
+      </c>
+      <c r="B133" t="s">
+        <v>217</v>
+      </c>
+      <c r="C133" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D133" t="s">
+        <v>218</v>
+      </c>
+      <c r="E133" t="s">
+        <v>224</v>
+      </c>
+      <c r="H133" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134">
+        <v>17</v>
+      </c>
+      <c r="B134" t="s">
+        <v>217</v>
+      </c>
+      <c r="C134" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D134" t="s">
+        <v>219</v>
+      </c>
+      <c r="E134" t="s">
+        <v>225</v>
+      </c>
+      <c r="H134" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A135">
+        <v>17</v>
+      </c>
+      <c r="B135" t="s">
+        <v>217</v>
+      </c>
+      <c r="C135" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D135" t="s">
+        <v>219</v>
+      </c>
+      <c r="E135" t="s">
+        <v>226</v>
+      </c>
+      <c r="H135" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136">
+        <v>17</v>
+      </c>
+      <c r="B136" t="s">
+        <v>217</v>
+      </c>
+      <c r="C136" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D136" t="s">
+        <v>220</v>
+      </c>
+      <c r="E136" t="s">
+        <v>227</v>
+      </c>
+      <c r="H136" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137">
+        <v>17</v>
+      </c>
+      <c r="B137" t="s">
+        <v>217</v>
+      </c>
+      <c r="C137" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D137" t="s">
+        <v>220</v>
+      </c>
+      <c r="E137" t="s">
+        <v>228</v>
+      </c>
+      <c r="H137" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>17</v>
+      </c>
+      <c r="B138" t="s">
+        <v>217</v>
+      </c>
+      <c r="C138" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D138" t="s">
+        <v>220</v>
+      </c>
+      <c r="E138" t="s">
+        <v>229</v>
+      </c>
+      <c r="H138" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>17</v>
+      </c>
+      <c r="B139" t="s">
+        <v>217</v>
+      </c>
+      <c r="C139" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D139" t="s">
+        <v>221</v>
+      </c>
+      <c r="E139" t="s">
+        <v>230</v>
+      </c>
+      <c r="H139" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>17</v>
+      </c>
+      <c r="B140" t="s">
+        <v>217</v>
+      </c>
+      <c r="C140" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D140" t="s">
+        <v>221</v>
+      </c>
+      <c r="E140" t="s">
+        <v>231</v>
+      </c>
+      <c r="H140" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>17</v>
+      </c>
+      <c r="B141" t="s">
+        <v>217</v>
+      </c>
+      <c r="C141" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D141" t="s">
+        <v>222</v>
+      </c>
+      <c r="E141" t="s">
+        <v>232</v>
+      </c>
+      <c r="H141" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142">
+        <v>17</v>
+      </c>
+      <c r="B142" t="s">
+        <v>217</v>
+      </c>
+      <c r="C142" s="1">
+        <v>46207</v>
+      </c>
+      <c r="D142" t="s">
+        <v>222</v>
+      </c>
+      <c r="E142" t="s">
+        <v>233</v>
+      </c>
+      <c r="H142" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
is an x a y hq polling results
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE131988-B5C8-4663-8685-439F1B39A242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E74F422-B8DF-4129-9C03-19F2AD5A5A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="258">
   <si>
     <t>option</t>
   </si>
@@ -762,6 +762,54 @@
   </si>
   <si>
     <t>Is cereal a soup?</t>
+  </si>
+  <si>
+    <t>Opposites</t>
+  </si>
+  <si>
+    <t>What's the opposite of fire?</t>
+  </si>
+  <si>
+    <t>What's the opposite of freezing?</t>
+  </si>
+  <si>
+    <t>What's the opposite of a question?</t>
+  </si>
+  <si>
+    <t>What's the opposite of an echo?</t>
+  </si>
+  <si>
+    <t>What's the opposite of a straight line?</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>No Fire</t>
+  </si>
+  <si>
+    <t>Melting</t>
+  </si>
+  <si>
+    <t>Boiling</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>Statement</t>
+  </si>
+  <si>
+    <t>Silence</t>
+  </si>
+  <si>
+    <t>Original Sound</t>
+  </si>
+  <si>
+    <t>Point</t>
+  </si>
+  <si>
+    <t>Curve</t>
   </si>
 </sst>
 </file>
@@ -1134,13 +1182,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H162"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
@@ -4632,8 +4680,11 @@
       <c r="E143" t="s">
         <v>236</v>
       </c>
+      <c r="F143">
+        <v>11</v>
+      </c>
       <c r="H143" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.25">
@@ -4652,8 +4703,11 @@
       <c r="E144" t="s">
         <v>237</v>
       </c>
+      <c r="F144">
+        <v>44</v>
+      </c>
       <c r="H144" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.25">
@@ -4672,8 +4726,11 @@
       <c r="E145" t="s">
         <v>236</v>
       </c>
+      <c r="F145">
+        <v>11</v>
+      </c>
       <c r="H145" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.25">
@@ -4692,8 +4749,11 @@
       <c r="E146" t="s">
         <v>237</v>
       </c>
+      <c r="F146">
+        <v>44</v>
+      </c>
       <c r="H146" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.25">
@@ -4712,8 +4772,11 @@
       <c r="E147" t="s">
         <v>236</v>
       </c>
+      <c r="F147">
+        <v>36</v>
+      </c>
       <c r="H147" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
@@ -4732,8 +4795,11 @@
       <c r="E148" t="s">
         <v>237</v>
       </c>
+      <c r="F148">
+        <v>19</v>
+      </c>
       <c r="H148" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.25">
@@ -4752,8 +4818,11 @@
       <c r="E149" t="s">
         <v>236</v>
       </c>
+      <c r="F149">
+        <v>27</v>
+      </c>
       <c r="H149" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
@@ -4772,8 +4841,11 @@
       <c r="E150" t="s">
         <v>237</v>
       </c>
+      <c r="F150">
+        <v>28</v>
+      </c>
       <c r="H150" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
@@ -4792,8 +4864,11 @@
       <c r="E151" t="s">
         <v>236</v>
       </c>
+      <c r="F151">
+        <v>8</v>
+      </c>
       <c r="H151" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
@@ -4812,7 +4887,210 @@
       <c r="E152" t="s">
         <v>237</v>
       </c>
+      <c r="F152">
+        <v>46</v>
+      </c>
       <c r="H152" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153">
+        <v>19</v>
+      </c>
+      <c r="B153" t="s">
+        <v>242</v>
+      </c>
+      <c r="C153" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D153" t="s">
+        <v>243</v>
+      </c>
+      <c r="E153" t="s">
+        <v>248</v>
+      </c>
+      <c r="H153" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154">
+        <v>19</v>
+      </c>
+      <c r="B154" t="s">
+        <v>242</v>
+      </c>
+      <c r="C154" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D154" t="s">
+        <v>243</v>
+      </c>
+      <c r="E154" t="s">
+        <v>249</v>
+      </c>
+      <c r="H154" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155">
+        <v>19</v>
+      </c>
+      <c r="B155" t="s">
+        <v>242</v>
+      </c>
+      <c r="C155" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D155" t="s">
+        <v>244</v>
+      </c>
+      <c r="E155" t="s">
+        <v>250</v>
+      </c>
+      <c r="H155" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156">
+        <v>19</v>
+      </c>
+      <c r="B156" t="s">
+        <v>242</v>
+      </c>
+      <c r="C156" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D156" t="s">
+        <v>244</v>
+      </c>
+      <c r="E156" t="s">
+        <v>251</v>
+      </c>
+      <c r="H156" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157">
+        <v>19</v>
+      </c>
+      <c r="B157" t="s">
+        <v>242</v>
+      </c>
+      <c r="C157" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D157" t="s">
+        <v>245</v>
+      </c>
+      <c r="E157" t="s">
+        <v>252</v>
+      </c>
+      <c r="H157" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158">
+        <v>19</v>
+      </c>
+      <c r="B158" t="s">
+        <v>242</v>
+      </c>
+      <c r="C158" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D158" t="s">
+        <v>245</v>
+      </c>
+      <c r="E158" t="s">
+        <v>253</v>
+      </c>
+      <c r="H158" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159">
+        <v>19</v>
+      </c>
+      <c r="B159" t="s">
+        <v>242</v>
+      </c>
+      <c r="C159" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D159" t="s">
+        <v>246</v>
+      </c>
+      <c r="E159" t="s">
+        <v>254</v>
+      </c>
+      <c r="H159" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160">
+        <v>19</v>
+      </c>
+      <c r="B160" t="s">
+        <v>242</v>
+      </c>
+      <c r="C160" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D160" t="s">
+        <v>246</v>
+      </c>
+      <c r="E160" t="s">
+        <v>255</v>
+      </c>
+      <c r="H160" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161">
+        <v>19</v>
+      </c>
+      <c r="B161" t="s">
+        <v>242</v>
+      </c>
+      <c r="C161" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D161" t="s">
+        <v>247</v>
+      </c>
+      <c r="E161" t="s">
+        <v>256</v>
+      </c>
+      <c r="H161" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162">
+        <v>19</v>
+      </c>
+      <c r="B162" t="s">
+        <v>242</v>
+      </c>
+      <c r="C162" s="1">
+        <v>46241</v>
+      </c>
+      <c r="D162" t="s">
+        <v>247</v>
+      </c>
+      <c r="E162" t="s">
+        <v>257</v>
+      </c>
+      <c r="H162" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
is x a y rtp polling results
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E74F422-B8DF-4129-9C03-19F2AD5A5A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0B84BD-F05E-442B-9C1D-8FB9FAE3318C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
@@ -4683,6 +4683,9 @@
       <c r="F143">
         <v>11</v>
       </c>
+      <c r="G143">
+        <v>7</v>
+      </c>
       <c r="H143" t="s">
         <v>148</v>
       </c>
@@ -4706,6 +4709,9 @@
       <c r="F144">
         <v>44</v>
       </c>
+      <c r="G144">
+        <v>29</v>
+      </c>
       <c r="H144" t="s">
         <v>148</v>
       </c>
@@ -4729,6 +4735,9 @@
       <c r="F145">
         <v>11</v>
       </c>
+      <c r="G145">
+        <v>8</v>
+      </c>
       <c r="H145" t="s">
         <v>148</v>
       </c>
@@ -4752,6 +4761,9 @@
       <c r="F146">
         <v>44</v>
       </c>
+      <c r="G146">
+        <v>28</v>
+      </c>
       <c r="H146" t="s">
         <v>148</v>
       </c>
@@ -4775,6 +4787,9 @@
       <c r="F147">
         <v>36</v>
       </c>
+      <c r="G147">
+        <v>19</v>
+      </c>
       <c r="H147" t="s">
         <v>148</v>
       </c>
@@ -4798,6 +4813,9 @@
       <c r="F148">
         <v>19</v>
       </c>
+      <c r="G148">
+        <v>17</v>
+      </c>
       <c r="H148" t="s">
         <v>148</v>
       </c>
@@ -4821,6 +4839,9 @@
       <c r="F149">
         <v>27</v>
       </c>
+      <c r="G149">
+        <v>20</v>
+      </c>
       <c r="H149" t="s">
         <v>148</v>
       </c>
@@ -4844,6 +4865,9 @@
       <c r="F150">
         <v>28</v>
       </c>
+      <c r="G150">
+        <v>16</v>
+      </c>
       <c r="H150" t="s">
         <v>148</v>
       </c>
@@ -4867,6 +4891,9 @@
       <c r="F151">
         <v>8</v>
       </c>
+      <c r="G151">
+        <v>8</v>
+      </c>
       <c r="H151" t="s">
         <v>148</v>
       </c>
@@ -4889,6 +4916,9 @@
       </c>
       <c r="F152">
         <v>46</v>
+      </c>
+      <c r="G152">
+        <v>29</v>
       </c>
       <c r="H152" t="s">
         <v>148</v>

</xml_diff>

<commit_message>
updated results for fair fare poll both locations
</commit_message>
<xml_diff>
--- a/whiteboardpollresults.xlsx
+++ b/whiteboardpollresults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mbrownin\GitHub - Local\thehallwaypoll\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB8565BE-D1B7-40EA-A50E-22F7F4CEF03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F21C0-06F8-499A-B908-312602C41141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-120" windowWidth="19440" windowHeight="14880" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="686" xr2:uid="{C0D0DBC0-4258-4C8D-AB0A-404DBED773F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="285">
   <si>
     <t>option</t>
   </si>
@@ -855,6 +855,42 @@
   </si>
   <si>
     <t>Blue Ribbon</t>
+  </si>
+  <si>
+    <t>Week Daze</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Favorite</t>
+  </si>
+  <si>
+    <t>Worst</t>
+  </si>
+  <si>
+    <t>Most Productive</t>
+  </si>
+  <si>
+    <t>Longest-Feeling</t>
   </si>
 </sst>
 </file>
@@ -1227,19 +1263,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C897EEBF-8298-48F4-84CA-7840A621B809}">
-  <dimension ref="A1:H172"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <dimension ref="A1:H200"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.41796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="10.83984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.68359375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.68359375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.68359375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.83984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>67</v>
       </c>
@@ -1265,7 +1301,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1288,7 +1324,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1311,7 +1347,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1334,7 +1370,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1357,7 +1393,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1380,7 +1416,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -1403,7 +1439,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
@@ -1426,7 +1462,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1449,7 +1485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1472,7 +1508,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1495,7 +1531,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
@@ -1518,7 +1554,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5</v>
       </c>
@@ -1541,7 +1577,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1564,7 +1600,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>5</v>
       </c>
@@ -1587,7 +1623,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>6</v>
       </c>
@@ -1610,7 +1646,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>6</v>
       </c>
@@ -1633,7 +1669,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>6</v>
       </c>
@@ -1656,7 +1692,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>6</v>
       </c>
@@ -1679,7 +1715,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>6</v>
       </c>
@@ -1702,7 +1738,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6</v>
       </c>
@@ -1725,7 +1761,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>6</v>
       </c>
@@ -1748,7 +1784,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>6</v>
       </c>
@@ -1771,7 +1807,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>7</v>
       </c>
@@ -1794,7 +1830,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>7</v>
       </c>
@@ -1817,7 +1853,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>7</v>
       </c>
@@ -1840,7 +1876,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>7</v>
       </c>
@@ -1863,7 +1899,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>7</v>
       </c>
@@ -1886,7 +1922,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>7</v>
       </c>
@@ -1909,7 +1945,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>7</v>
       </c>
@@ -1932,7 +1968,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>7</v>
       </c>
@@ -1955,7 +1991,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>8</v>
       </c>
@@ -1978,7 +2014,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>8</v>
       </c>
@@ -2001,7 +2037,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>8</v>
       </c>
@@ -2024,7 +2060,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>8</v>
       </c>
@@ -2047,7 +2083,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>8</v>
       </c>
@@ -2070,7 +2106,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>8</v>
       </c>
@@ -2093,7 +2129,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>8</v>
       </c>
@@ -2116,7 +2152,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>8</v>
       </c>
@@ -2139,7 +2175,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>8</v>
       </c>
@@ -2162,7 +2198,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>8</v>
       </c>
@@ -2185,7 +2221,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>9</v>
       </c>
@@ -2208,7 +2244,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>9</v>
       </c>
@@ -2231,7 +2267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>9</v>
       </c>
@@ -2254,7 +2290,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>9</v>
       </c>
@@ -2277,7 +2313,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>9</v>
       </c>
@@ -2300,7 +2336,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>9</v>
       </c>
@@ -2323,7 +2359,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>9</v>
       </c>
@@ -2346,7 +2382,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>9</v>
       </c>
@@ -2369,7 +2405,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>9</v>
       </c>
@@ -2392,7 +2428,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>9</v>
       </c>
@@ -2415,7 +2451,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10</v>
       </c>
@@ -2438,7 +2474,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10</v>
       </c>
@@ -2461,7 +2497,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10</v>
       </c>
@@ -2484,7 +2520,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10</v>
       </c>
@@ -2507,7 +2543,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10</v>
       </c>
@@ -2530,7 +2566,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>10</v>
       </c>
@@ -2553,7 +2589,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>10</v>
       </c>
@@ -2576,7 +2612,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10</v>
       </c>
@@ -2599,7 +2635,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>10</v>
       </c>
@@ -2622,7 +2658,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10</v>
       </c>
@@ -2645,7 +2681,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>11</v>
       </c>
@@ -2668,7 +2704,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>11</v>
       </c>
@@ -2691,7 +2727,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>11</v>
       </c>
@@ -2714,7 +2750,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>11</v>
       </c>
@@ -2737,7 +2773,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>11</v>
       </c>
@@ -2760,7 +2796,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>11</v>
       </c>
@@ -2783,7 +2819,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>11</v>
       </c>
@@ -2806,7 +2842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>11</v>
       </c>
@@ -2829,7 +2865,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>11</v>
       </c>
@@ -2852,7 +2888,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>11</v>
       </c>
@@ -2875,7 +2911,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>11</v>
       </c>
@@ -2898,7 +2934,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>11</v>
       </c>
@@ -2921,7 +2957,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>11</v>
       </c>
@@ -2944,7 +2980,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>11</v>
       </c>
@@ -2967,7 +3003,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>12</v>
       </c>
@@ -2993,7 +3029,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>12</v>
       </c>
@@ -3019,7 +3055,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>12</v>
       </c>
@@ -3045,7 +3081,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>12</v>
       </c>
@@ -3071,7 +3107,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>12</v>
       </c>
@@ -3097,7 +3133,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>12</v>
       </c>
@@ -3123,7 +3159,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>12</v>
       </c>
@@ -3149,7 +3185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>12</v>
       </c>
@@ -3175,7 +3211,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>13</v>
       </c>
@@ -3201,7 +3237,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>13</v>
       </c>
@@ -3227,7 +3263,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>13</v>
       </c>
@@ -3253,7 +3289,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>13</v>
       </c>
@@ -3279,7 +3315,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>13</v>
       </c>
@@ -3305,7 +3341,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>13</v>
       </c>
@@ -3331,7 +3367,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>13</v>
       </c>
@@ -3357,7 +3393,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>13</v>
       </c>
@@ -3383,7 +3419,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>13</v>
       </c>
@@ -3409,7 +3445,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>13</v>
       </c>
@@ -3435,7 +3471,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>13</v>
       </c>
@@ -3461,7 +3497,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>13</v>
       </c>
@@ -3487,7 +3523,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>13</v>
       </c>
@@ -3513,7 +3549,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>13</v>
       </c>
@@ -3539,7 +3575,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>14</v>
       </c>
@@ -3565,7 +3601,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>14</v>
       </c>
@@ -3591,7 +3627,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>14</v>
       </c>
@@ -3617,7 +3653,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>14</v>
       </c>
@@ -3643,7 +3679,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>14</v>
       </c>
@@ -3669,7 +3705,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>14</v>
       </c>
@@ -3695,7 +3731,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>14</v>
       </c>
@@ -3721,7 +3757,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>14</v>
       </c>
@@ -3747,7 +3783,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>14</v>
       </c>
@@ -3773,7 +3809,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>14</v>
       </c>
@@ -3799,7 +3835,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>15</v>
       </c>
@@ -3825,7 +3861,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>15</v>
       </c>
@@ -3851,7 +3887,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>15</v>
       </c>
@@ -3877,7 +3913,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>15</v>
       </c>
@@ -3903,7 +3939,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>15</v>
       </c>
@@ -3929,7 +3965,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>15</v>
       </c>
@@ -3955,7 +3991,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>15</v>
       </c>
@@ -3981,7 +4017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>15</v>
       </c>
@@ -4007,7 +4043,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>15</v>
       </c>
@@ -4033,7 +4069,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>15</v>
       </c>
@@ -4059,7 +4095,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>15</v>
       </c>
@@ -4085,7 +4121,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>15</v>
       </c>
@@ -4111,7 +4147,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>15</v>
       </c>
@@ -4137,7 +4173,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>15</v>
       </c>
@@ -4163,7 +4199,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>16</v>
       </c>
@@ -4189,7 +4225,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>16</v>
       </c>
@@ -4215,7 +4251,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>16</v>
       </c>
@@ -4241,7 +4277,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>16</v>
       </c>
@@ -4267,7 +4303,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>16</v>
       </c>
@@ -4293,7 +4329,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>16</v>
       </c>
@@ -4319,7 +4355,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>16</v>
       </c>
@@ -4345,7 +4381,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>16</v>
       </c>
@@ -4371,7 +4407,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>16</v>
       </c>
@@ -4397,7 +4433,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>16</v>
       </c>
@@ -4423,7 +4459,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>17</v>
       </c>
@@ -4449,7 +4485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>17</v>
       </c>
@@ -4475,7 +4511,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>17</v>
       </c>
@@ -4501,7 +4537,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>17</v>
       </c>
@@ -4527,7 +4563,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>17</v>
       </c>
@@ -4553,7 +4589,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>17</v>
       </c>
@@ -4579,7 +4615,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>17</v>
       </c>
@@ -4605,7 +4641,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>17</v>
       </c>
@@ -4631,7 +4667,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>17</v>
       </c>
@@ -4657,7 +4693,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>17</v>
       </c>
@@ -4683,7 +4719,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>17</v>
       </c>
@@ -4709,7 +4745,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>18</v>
       </c>
@@ -4735,7 +4771,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>18</v>
       </c>
@@ -4761,7 +4797,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>18</v>
       </c>
@@ -4787,7 +4823,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>18</v>
       </c>
@@ -4813,7 +4849,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>18</v>
       </c>
@@ -4839,7 +4875,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>18</v>
       </c>
@@ -4865,7 +4901,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>18</v>
       </c>
@@ -4891,7 +4927,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>18</v>
       </c>
@@ -4917,7 +4953,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>18</v>
       </c>
@@ -4943,7 +4979,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>18</v>
       </c>
@@ -4969,7 +5005,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>19</v>
       </c>
@@ -4995,7 +5031,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>19</v>
       </c>
@@ -5021,7 +5057,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>19</v>
       </c>
@@ -5047,7 +5083,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>19</v>
       </c>
@@ -5073,7 +5109,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>19</v>
       </c>
@@ -5099,7 +5135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>19</v>
       </c>
@@ -5125,7 +5161,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>19</v>
       </c>
@@ -5151,7 +5187,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>19</v>
       </c>
@@ -5177,7 +5213,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>19</v>
       </c>
@@ -5203,7 +5239,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>19</v>
       </c>
@@ -5229,7 +5265,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>20</v>
       </c>
@@ -5245,11 +5281,17 @@
       <c r="E163" t="s">
         <v>263</v>
       </c>
+      <c r="F163">
+        <v>23</v>
+      </c>
+      <c r="G163">
+        <v>14</v>
+      </c>
       <c r="H163" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>20</v>
       </c>
@@ -5265,11 +5307,17 @@
       <c r="E164" t="s">
         <v>264</v>
       </c>
+      <c r="F164">
+        <v>17</v>
+      </c>
+      <c r="G164">
+        <v>7</v>
+      </c>
       <c r="H164" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>20</v>
       </c>
@@ -5285,11 +5333,17 @@
       <c r="E165" t="s">
         <v>265</v>
       </c>
+      <c r="F165">
+        <v>32</v>
+      </c>
+      <c r="G165">
+        <v>13</v>
+      </c>
       <c r="H165" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>20</v>
       </c>
@@ -5305,11 +5359,17 @@
       <c r="E166" t="s">
         <v>266</v>
       </c>
+      <c r="F166">
+        <v>10</v>
+      </c>
+      <c r="G166">
+        <v>9</v>
+      </c>
       <c r="H166" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>20</v>
       </c>
@@ -5325,11 +5385,17 @@
       <c r="E167" t="s">
         <v>267</v>
       </c>
+      <c r="F167">
+        <v>29</v>
+      </c>
+      <c r="G167">
+        <v>15</v>
+      </c>
       <c r="H167" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>20</v>
       </c>
@@ -5345,11 +5411,17 @@
       <c r="E168" t="s">
         <v>268</v>
       </c>
+      <c r="F168">
+        <v>10</v>
+      </c>
+      <c r="G168">
+        <v>7</v>
+      </c>
       <c r="H168" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>20</v>
       </c>
@@ -5365,11 +5437,17 @@
       <c r="E169" t="s">
         <v>269</v>
       </c>
+      <c r="F169">
+        <v>30</v>
+      </c>
+      <c r="G169">
+        <v>17</v>
+      </c>
       <c r="H169" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>20</v>
       </c>
@@ -5385,11 +5463,17 @@
       <c r="E170" t="s">
         <v>270</v>
       </c>
+      <c r="F170">
+        <v>12</v>
+      </c>
+      <c r="G170">
+        <v>5</v>
+      </c>
       <c r="H170" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>20</v>
       </c>
@@ -5405,11 +5489,17 @@
       <c r="E171" t="s">
         <v>271</v>
       </c>
+      <c r="F171">
+        <v>29</v>
+      </c>
+      <c r="G171">
+        <v>20</v>
+      </c>
       <c r="H171" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>20</v>
       </c>
@@ -5425,7 +5515,573 @@
       <c r="E172" t="s">
         <v>272</v>
       </c>
+      <c r="F172">
+        <v>12</v>
+      </c>
+      <c r="G172">
+        <v>2</v>
+      </c>
       <c r="H172" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173">
+        <v>21</v>
+      </c>
+      <c r="B173" t="s">
+        <v>273</v>
+      </c>
+      <c r="C173" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D173" t="s">
+        <v>281</v>
+      </c>
+      <c r="E173" t="s">
+        <v>274</v>
+      </c>
+      <c r="H173" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174">
+        <v>21</v>
+      </c>
+      <c r="B174" t="s">
+        <v>273</v>
+      </c>
+      <c r="C174" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D174" t="s">
+        <v>281</v>
+      </c>
+      <c r="E174" t="s">
+        <v>275</v>
+      </c>
+      <c r="H174" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175">
+        <v>21</v>
+      </c>
+      <c r="B175" t="s">
+        <v>273</v>
+      </c>
+      <c r="C175" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D175" t="s">
+        <v>281</v>
+      </c>
+      <c r="E175" t="s">
+        <v>276</v>
+      </c>
+      <c r="H175" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176">
+        <v>21</v>
+      </c>
+      <c r="B176" t="s">
+        <v>273</v>
+      </c>
+      <c r="C176" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D176" t="s">
+        <v>281</v>
+      </c>
+      <c r="E176" t="s">
+        <v>277</v>
+      </c>
+      <c r="H176" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177">
+        <v>21</v>
+      </c>
+      <c r="B177" t="s">
+        <v>273</v>
+      </c>
+      <c r="C177" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D177" t="s">
+        <v>281</v>
+      </c>
+      <c r="E177" t="s">
+        <v>278</v>
+      </c>
+      <c r="H177" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178">
+        <v>21</v>
+      </c>
+      <c r="B178" t="s">
+        <v>273</v>
+      </c>
+      <c r="C178" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D178" t="s">
+        <v>281</v>
+      </c>
+      <c r="E178" t="s">
+        <v>279</v>
+      </c>
+      <c r="H178" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>21</v>
+      </c>
+      <c r="B179" t="s">
+        <v>273</v>
+      </c>
+      <c r="C179" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D179" t="s">
+        <v>281</v>
+      </c>
+      <c r="E179" t="s">
+        <v>280</v>
+      </c>
+      <c r="H179" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>21</v>
+      </c>
+      <c r="B180" t="s">
+        <v>273</v>
+      </c>
+      <c r="C180" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D180" t="s">
+        <v>282</v>
+      </c>
+      <c r="E180" t="s">
+        <v>274</v>
+      </c>
+      <c r="H180" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>21</v>
+      </c>
+      <c r="B181" t="s">
+        <v>273</v>
+      </c>
+      <c r="C181" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D181" t="s">
+        <v>282</v>
+      </c>
+      <c r="E181" t="s">
+        <v>275</v>
+      </c>
+      <c r="H181" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>21</v>
+      </c>
+      <c r="B182" t="s">
+        <v>273</v>
+      </c>
+      <c r="C182" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D182" t="s">
+        <v>282</v>
+      </c>
+      <c r="E182" t="s">
+        <v>276</v>
+      </c>
+      <c r="H182" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>21</v>
+      </c>
+      <c r="B183" t="s">
+        <v>273</v>
+      </c>
+      <c r="C183" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D183" t="s">
+        <v>282</v>
+      </c>
+      <c r="E183" t="s">
+        <v>277</v>
+      </c>
+      <c r="H183" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>21</v>
+      </c>
+      <c r="B184" t="s">
+        <v>273</v>
+      </c>
+      <c r="C184" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D184" t="s">
+        <v>282</v>
+      </c>
+      <c r="E184" t="s">
+        <v>278</v>
+      </c>
+      <c r="H184" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>21</v>
+      </c>
+      <c r="B185" t="s">
+        <v>273</v>
+      </c>
+      <c r="C185" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D185" t="s">
+        <v>282</v>
+      </c>
+      <c r="E185" t="s">
+        <v>279</v>
+      </c>
+      <c r="H185" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>21</v>
+      </c>
+      <c r="B186" t="s">
+        <v>273</v>
+      </c>
+      <c r="C186" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D186" t="s">
+        <v>282</v>
+      </c>
+      <c r="E186" t="s">
+        <v>280</v>
+      </c>
+      <c r="H186" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>21</v>
+      </c>
+      <c r="B187" t="s">
+        <v>273</v>
+      </c>
+      <c r="C187" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D187" t="s">
+        <v>283</v>
+      </c>
+      <c r="E187" t="s">
+        <v>274</v>
+      </c>
+      <c r="H187" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>21</v>
+      </c>
+      <c r="B188" t="s">
+        <v>273</v>
+      </c>
+      <c r="C188" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D188" t="s">
+        <v>283</v>
+      </c>
+      <c r="E188" t="s">
+        <v>275</v>
+      </c>
+      <c r="H188" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>21</v>
+      </c>
+      <c r="B189" t="s">
+        <v>273</v>
+      </c>
+      <c r="C189" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D189" t="s">
+        <v>283</v>
+      </c>
+      <c r="E189" t="s">
+        <v>276</v>
+      </c>
+      <c r="H189" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>21</v>
+      </c>
+      <c r="B190" t="s">
+        <v>273</v>
+      </c>
+      <c r="C190" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D190" t="s">
+        <v>283</v>
+      </c>
+      <c r="E190" t="s">
+        <v>277</v>
+      </c>
+      <c r="H190" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>21</v>
+      </c>
+      <c r="B191" t="s">
+        <v>273</v>
+      </c>
+      <c r="C191" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D191" t="s">
+        <v>283</v>
+      </c>
+      <c r="E191" t="s">
+        <v>278</v>
+      </c>
+      <c r="H191" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>21</v>
+      </c>
+      <c r="B192" t="s">
+        <v>273</v>
+      </c>
+      <c r="C192" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D192" t="s">
+        <v>283</v>
+      </c>
+      <c r="E192" t="s">
+        <v>279</v>
+      </c>
+      <c r="H192" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>21</v>
+      </c>
+      <c r="B193" t="s">
+        <v>273</v>
+      </c>
+      <c r="C193" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D193" t="s">
+        <v>283</v>
+      </c>
+      <c r="E193" t="s">
+        <v>280</v>
+      </c>
+      <c r="H193" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>21</v>
+      </c>
+      <c r="B194" t="s">
+        <v>273</v>
+      </c>
+      <c r="C194" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D194" t="s">
+        <v>284</v>
+      </c>
+      <c r="E194" t="s">
+        <v>274</v>
+      </c>
+      <c r="H194" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>21</v>
+      </c>
+      <c r="B195" t="s">
+        <v>273</v>
+      </c>
+      <c r="C195" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D195" t="s">
+        <v>284</v>
+      </c>
+      <c r="E195" t="s">
+        <v>275</v>
+      </c>
+      <c r="H195" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A196">
+        <v>21</v>
+      </c>
+      <c r="B196" t="s">
+        <v>273</v>
+      </c>
+      <c r="C196" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D196" t="s">
+        <v>284</v>
+      </c>
+      <c r="E196" t="s">
+        <v>276</v>
+      </c>
+      <c r="H196" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>21</v>
+      </c>
+      <c r="B197" t="s">
+        <v>273</v>
+      </c>
+      <c r="C197" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D197" t="s">
+        <v>284</v>
+      </c>
+      <c r="E197" t="s">
+        <v>277</v>
+      </c>
+      <c r="H197" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>21</v>
+      </c>
+      <c r="B198" t="s">
+        <v>273</v>
+      </c>
+      <c r="C198" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D198" t="s">
+        <v>284</v>
+      </c>
+      <c r="E198" t="s">
+        <v>278</v>
+      </c>
+      <c r="H198" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>21</v>
+      </c>
+      <c r="B199" t="s">
+        <v>273</v>
+      </c>
+      <c r="C199" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D199" t="s">
+        <v>284</v>
+      </c>
+      <c r="E199" t="s">
+        <v>279</v>
+      </c>
+      <c r="H199" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>21</v>
+      </c>
+      <c r="B200" t="s">
+        <v>273</v>
+      </c>
+      <c r="C200" s="1">
+        <v>46269</v>
+      </c>
+      <c r="D200" t="s">
+        <v>284</v>
+      </c>
+      <c r="E200" t="s">
+        <v>280</v>
+      </c>
+      <c r="H200" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>